<commit_message>
Improvements of the preregistration
</commit_message>
<xml_diff>
--- a/AllEndParameters.xlsx
+++ b/AllEndParameters.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:J137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,25 +436,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>H0</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>E0</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
@@ -467,21 +482,30 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.216026239091676</v>
+        <v>0.008951417552238038</v>
       </c>
       <c r="C2" t="n">
+        <v>0.006643163829489937</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.006101429295882835</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.3111132988228749</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>0.01615005793310728</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
+        <v>0.004882801652277004</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.1312290331861811</v>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="n">
         <v>0.5427127809982065</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>0.6228255112231958</v>
       </c>
     </row>
@@ -492,21 +516,30 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1832236078726236</v>
+        <v>0.007827425236935319</v>
       </c>
       <c r="C3" t="n">
+        <v>0.005354459529693851</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.004648320375074087</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.2638373501615357</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>0.01268003312630957</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
+        <v>0.005980798887152796</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.1218912572355742</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="n">
         <v>0.4660107893664037</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>0.511749012459412</v>
       </c>
     </row>
@@ -517,21 +550,30 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2110615495774004</v>
+        <v>0.008887477735955917</v>
       </c>
       <c r="C4" t="n">
+        <v>0.006513019622662825</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.005915096104301936</v>
+      </c>
+      <c r="E4" t="n">
         <v>0.3040218545891681</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>0.01610366844039917</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
+        <v>0.004720147299524383</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.1354698069234266</v>
       </c>
-      <c r="F4" t="n">
+      <c r="I4" t="n">
         <v>0.523575280077599</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
         <v>0.6080264944059606</v>
       </c>
     </row>
@@ -542,21 +584,30 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1825789458387865</v>
+        <v>0.007844950321246942</v>
       </c>
       <c r="C5" t="n">
+        <v>0.005358393936182266</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.004651775959678513</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.262895130892931</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>0.01279765592768531</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
+        <v>0.006104772457915853</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.1239051995433976</v>
       </c>
-      <c r="F5" t="n">
+      <c r="I5" t="n">
         <v>0.4629955496295349</v>
       </c>
-      <c r="G5" t="n">
+      <c r="J5" t="n">
         <v>0.508804468670378</v>
       </c>
     </row>
@@ -567,21 +618,30 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1947159467944987</v>
+        <v>0.008029461129619371</v>
       </c>
       <c r="C6" t="n">
+        <v>0.005670855782962394</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.004996260427411433</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.2802985048151565</v>
       </c>
-      <c r="D6" t="n">
+      <c r="F6" t="n">
         <v>0.01258189175420775</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
+        <v>0.003582133383236947</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.1113806749053137</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="n">
         <v>0.5027593340292468</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>0.5546341523523156</v>
       </c>
     </row>
@@ -592,21 +652,30 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1672928237314504</v>
+        <v>0.00684908675779922</v>
       </c>
       <c r="C7" t="n">
+        <v>0.004454919885469976</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.003642655864293197</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.2408647102852253</v>
       </c>
-      <c r="D7" t="n">
+      <c r="F7" t="n">
         <v>0.01082403318615315</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
+        <v>0.003886250433339808</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.1145014619849383</v>
       </c>
-      <c r="F7" t="n">
+      <c r="I7" t="n">
         <v>0.4248094780487133</v>
       </c>
-      <c r="G7" t="n">
+      <c r="J7" t="n">
         <v>0.4646303696604731</v>
       </c>
     </row>
@@ -617,21 +686,30 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1967337981809544</v>
+        <v>0.008076713087947079</v>
       </c>
       <c r="C8" t="n">
+        <v>0.005738729340569819</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.005082491538748863</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.2831975485891929</v>
       </c>
-      <c r="D8" t="n">
+      <c r="F8" t="n">
         <v>0.01278478456397261</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
+        <v>0.003524448318773375</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.1119732221313501</v>
       </c>
-      <c r="F8" t="n">
+      <c r="I8" t="n">
         <v>0.5075462952245926</v>
       </c>
-      <c r="G8" t="n">
+      <c r="J8" t="n">
         <v>0.5611190934975623</v>
       </c>
     </row>
@@ -642,21 +720,30 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.164929215088086</v>
+        <v>0.006716280243098316</v>
       </c>
       <c r="C9" t="n">
+        <v>0.004331334272996243</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.003504266451684443</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.2373896757695489</v>
       </c>
-      <c r="D9" t="n">
+      <c r="F9" t="n">
         <v>0.01067761889105638</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
+        <v>0.003624001987124435</v>
+      </c>
+      <c r="H9" t="n">
         <v>0.1152712059298999</v>
       </c>
-      <c r="F9" t="n">
+      <c r="I9" t="n">
         <v>0.4169959935893893</v>
       </c>
-      <c r="G9" t="n">
+      <c r="J9" t="n">
         <v>0.4574968787814851</v>
       </c>
     </row>
@@ -667,21 +754,30 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2166839246274135</v>
+        <v>0.009191087915265704</v>
       </c>
       <c r="C10" t="n">
+        <v>0.006835136289179387</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.006343293727948548</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.312107175518941</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
         <v>0.01613030789627663</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
+        <v>0.006604038257104305</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.1298326861678777</v>
       </c>
-      <c r="F10" t="n">
+      <c r="I10" t="n">
         <v>0.5481787247909533</v>
       </c>
-      <c r="G10" t="n">
+      <c r="J10" t="n">
         <v>0.6226456113144255</v>
       </c>
     </row>
@@ -692,21 +788,30 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1865416818270735</v>
+        <v>0.007961472076232433</v>
       </c>
       <c r="C11" t="n">
+        <v>0.005485319345697597</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.004770870531022391</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.2686530261390253</v>
       </c>
-      <c r="D11" t="n">
+      <c r="F11" t="n">
         <v>0.01309363917850703</v>
       </c>
-      <c r="E11" t="n">
+      <c r="G11" t="n">
+        <v>0.006028087869660126</v>
+      </c>
+      <c r="H11" t="n">
         <v>0.1235519817347275</v>
       </c>
-      <c r="F11" t="n">
+      <c r="I11" t="n">
         <v>0.472943348345983</v>
       </c>
-      <c r="G11" t="n">
+      <c r="J11" t="n">
         <v>0.5229614813016559</v>
       </c>
     </row>
@@ -717,21 +822,30 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.218513245906913</v>
+        <v>0.009322631252452848</v>
       </c>
       <c r="C12" t="n">
+        <v>0.006954747584352194</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.006460133267100597</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.3147106944671311</v>
       </c>
-      <c r="D12" t="n">
+      <c r="F12" t="n">
         <v>0.01596973481920821</v>
       </c>
-      <c r="E12" t="n">
+      <c r="G12" t="n">
+        <v>0.006360608780822296</v>
+      </c>
+      <c r="H12" t="n">
         <v>0.1266529900638307</v>
       </c>
-      <c r="F12" t="n">
+      <c r="I12" t="n">
         <v>0.5569010559161129</v>
       </c>
-      <c r="G12" t="n">
+      <c r="J12" t="n">
         <v>0.6280764244782114</v>
       </c>
     </row>
@@ -742,21 +856,30 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.185809138257377</v>
+        <v>0.007964548831876771</v>
       </c>
       <c r="C13" t="n">
+        <v>0.005477174469852599</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.004760370733311644</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.2676382448138035</v>
       </c>
-      <c r="D13" t="n">
+      <c r="F13" t="n">
         <v>0.01314525872177437</v>
       </c>
-      <c r="E13" t="n">
+      <c r="G13" t="n">
+        <v>0.00606867785207475</v>
+      </c>
+      <c r="H13" t="n">
         <v>0.1248629712953642</v>
       </c>
-      <c r="F13" t="n">
+      <c r="I13" t="n">
         <v>0.4694377596778758</v>
       </c>
-      <c r="G13" t="n">
+      <c r="J13" t="n">
         <v>0.5207701574056377</v>
       </c>
     </row>
@@ -767,21 +890,30 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.2172938798030039</v>
+        <v>0.009496527729323372</v>
       </c>
       <c r="C14" t="n">
+        <v>0.007107956195812294</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.006667430479789428</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.3129784901755389</v>
       </c>
-      <c r="D14" t="n">
+      <c r="F14" t="n">
         <v>0.01509134706351103</v>
       </c>
-      <c r="E14" t="n">
+      <c r="G14" t="n">
+        <v>0.005710483601031855</v>
+      </c>
+      <c r="H14" t="n">
         <v>0.1187724184746507</v>
       </c>
-      <c r="F14" t="n">
+      <c r="I14" t="n">
         <v>0.5617694290981515</v>
       </c>
-      <c r="G14" t="n">
+      <c r="J14" t="n">
         <v>0.6236852954216845</v>
       </c>
     </row>
@@ -792,21 +924,30 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1868468958048795</v>
+        <v>0.008142482081100575</v>
       </c>
       <c r="C15" t="n">
+        <v>0.005633259922848116</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.004966092442132396</v>
+      </c>
+      <c r="E15" t="n">
         <v>0.2691282475481587</v>
       </c>
-      <c r="D15" t="n">
+      <c r="F15" t="n">
         <v>0.01274979981809723</v>
       </c>
-      <c r="E15" t="n">
+      <c r="G15" t="n">
+        <v>0.006590579003254088</v>
+      </c>
+      <c r="H15" t="n">
         <v>0.1186524293510159</v>
       </c>
-      <c r="F15" t="n">
+      <c r="I15" t="n">
         <v>0.4816689475211184</v>
       </c>
-      <c r="G15" t="n">
+      <c r="J15" t="n">
         <v>0.5210367086248769</v>
       </c>
     </row>
@@ -817,21 +958,30 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.2096522014120281</v>
+        <v>0.00919214203967009</v>
       </c>
       <c r="C16" t="n">
+        <v>0.006742405708155812</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.006179250989382432</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.3019603796572657</v>
       </c>
-      <c r="D16" t="n">
+      <c r="F16" t="n">
         <v>0.01452419308152283</v>
       </c>
-      <c r="E16" t="n">
+      <c r="G16" t="n">
+        <v>0.004609253219068597</v>
+      </c>
+      <c r="H16" t="n">
         <v>0.1193699414540482</v>
       </c>
-      <c r="F16" t="n">
+      <c r="I16" t="n">
         <v>0.5385360636631181</v>
       </c>
-      <c r="G16" t="n">
+      <c r="J16" t="n">
         <v>0.6006024023472278</v>
       </c>
     </row>
@@ -842,21 +992,30 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.1840756587708758</v>
+        <v>0.008035692001401558</v>
       </c>
       <c r="C17" t="n">
+        <v>0.005511155222706843</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.004810012650851755</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.2651159058378642</v>
       </c>
-      <c r="D17" t="n">
+      <c r="F17" t="n">
         <v>0.01259042972958943</v>
       </c>
-      <c r="E17" t="n">
+      <c r="G17" t="n">
+        <v>0.006384527287544652</v>
+      </c>
+      <c r="H17" t="n">
         <v>0.1194444717502028</v>
       </c>
-      <c r="F17" t="n">
+      <c r="I17" t="n">
         <v>0.47331168601227</v>
       </c>
-      <c r="G17" t="n">
+      <c r="J17" t="n">
         <v>0.5119994754239673</v>
       </c>
     </row>
@@ -867,21 +1026,30 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.1927942101625485</v>
+        <v>0.007323848600783188</v>
       </c>
       <c r="C18" t="n">
+        <v>0.005121947775021266</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.004448135783702388</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.2776534903777834</v>
       </c>
-      <c r="D18" t="n">
+      <c r="F18" t="n">
         <v>0.0134741359378533</v>
       </c>
-      <c r="E18" t="n">
+      <c r="G18" t="n">
+        <v>0.003479188834899137</v>
+      </c>
+      <c r="H18" t="n">
         <v>0.1233155734700789</v>
       </c>
-      <c r="F18" t="n">
+      <c r="I18" t="n">
         <v>0.4834510693194896</v>
       </c>
-      <c r="G18" t="n">
+      <c r="J18" t="n">
         <v>0.5504163371198718</v>
       </c>
     </row>
@@ -892,21 +1060,30 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.1698748524744804</v>
+        <v>0.006439450125720734</v>
       </c>
       <c r="C19" t="n">
+        <v>0.004220386675590976</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.003470212325431503</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.2446604409476694</v>
       </c>
-      <c r="D19" t="n">
+      <c r="F19" t="n">
         <v>0.01120121827895115</v>
       </c>
-      <c r="E19" t="n">
+      <c r="G19" t="n">
+        <v>0.003833362085579621</v>
+      </c>
+      <c r="H19" t="n">
         <v>0.117127027722989</v>
       </c>
-      <c r="F19" t="n">
+      <c r="I19" t="n">
         <v>0.4269509163059212</v>
       </c>
-      <c r="G19" t="n">
+      <c r="J19" t="n">
         <v>0.4753881967361854</v>
       </c>
     </row>
@@ -917,21 +1094,30 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.1896916347378046</v>
+        <v>0.007381244134466307</v>
       </c>
       <c r="C20" t="n">
+        <v>0.005128506571488517</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.004438590217620726</v>
+      </c>
+      <c r="E20" t="n">
         <v>0.2731530179468055</v>
       </c>
-      <c r="D20" t="n">
+      <c r="F20" t="n">
         <v>0.01270853378283794</v>
       </c>
-      <c r="E20" t="n">
+      <c r="G20" t="n">
+        <v>0.003252216640537761</v>
+      </c>
+      <c r="H20" t="n">
         <v>0.117128231052045</v>
       </c>
-      <c r="F20" t="n">
+      <c r="I20" t="n">
         <v>0.4815371470856425</v>
       </c>
-      <c r="G20" t="n">
+      <c r="J20" t="n">
         <v>0.540000882093131</v>
       </c>
     </row>
@@ -942,21 +1128,30 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.1694284789608485</v>
+        <v>0.006499136236380645</v>
       </c>
       <c r="C21" t="n">
+        <v>0.004257844065455772</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.003508438854763438</v>
+      </c>
+      <c r="E21" t="n">
         <v>0.2439309712743911</v>
       </c>
-      <c r="D21" t="n">
+      <c r="F21" t="n">
         <v>0.01126638494299079</v>
       </c>
-      <c r="E21" t="n">
+      <c r="G21" t="n">
+        <v>0.003998657957534526</v>
+      </c>
+      <c r="H21" t="n">
         <v>0.1186643957208108</v>
       </c>
-      <c r="F21" t="n">
+      <c r="I21" t="n">
         <v>0.4247217579041031</v>
       </c>
-      <c r="G21" t="n">
+      <c r="J21" t="n">
         <v>0.473351067065804</v>
       </c>
     </row>
@@ -967,21 +1162,30 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.1816178128267908</v>
+        <v>0.008283981817211175</v>
       </c>
       <c r="C22" t="n">
+        <v>0.005594311714314828</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.004659973717051727</v>
+      </c>
+      <c r="E22" t="n">
         <v>0.2616040980601079</v>
       </c>
-      <c r="D22" t="n">
+      <c r="F22" t="n">
         <v>0.01329272437762484</v>
       </c>
-      <c r="E22" t="n">
+      <c r="G22" t="n">
+        <v>0.002925618480786542</v>
+      </c>
+      <c r="H22" t="n">
         <v>0.1336022665490282</v>
       </c>
-      <c r="F22" t="n">
+      <c r="I22" t="n">
         <v>0.4400891061469429</v>
       </c>
-      <c r="G22" t="n">
+      <c r="J22" t="n">
         <v>0.5167955666952184</v>
       </c>
     </row>
@@ -992,21 +1196,30 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.1596762393252448</v>
+        <v>0.007313837591805056</v>
       </c>
       <c r="C23" t="n">
+        <v>0.004617953671141227</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.003624443917043648</v>
+      </c>
+      <c r="E23" t="n">
         <v>0.229863832257019</v>
       </c>
-      <c r="D23" t="n">
+      <c r="F23" t="n">
         <v>0.01082115692284296</v>
       </c>
-      <c r="E23" t="n">
+      <c r="G23" t="n">
+        <v>0.002716016087544049</v>
+      </c>
+      <c r="H23" t="n">
         <v>0.1239886054775259</v>
       </c>
-      <c r="F23" t="n">
+      <c r="I23" t="n">
         <v>0.3916484642015665</v>
       </c>
-      <c r="G23" t="n">
+      <c r="J23" t="n">
         <v>0.4427097189254528</v>
       </c>
     </row>
@@ -1017,21 +1230,30 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.1814820509444049</v>
+        <v>0.008300175330556592</v>
       </c>
       <c r="C24" t="n">
+        <v>0.005604172413737068</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.004667422125521894</v>
+      </c>
+      <c r="E24" t="n">
         <v>0.2614460328056055</v>
       </c>
-      <c r="D24" t="n">
+      <c r="F24" t="n">
         <v>0.01316632105799156</v>
       </c>
-      <c r="E24" t="n">
+      <c r="G24" t="n">
+        <v>0.002886176636487681</v>
+      </c>
+      <c r="H24" t="n">
         <v>0.131902065815708</v>
       </c>
-      <c r="F24" t="n">
+      <c r="I24" t="n">
         <v>0.4414719582842397</v>
       </c>
-      <c r="G24" t="n">
+      <c r="J24" t="n">
         <v>0.5163660850942648</v>
       </c>
     </row>
@@ -1042,21 +1264,30 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.1589416496489766</v>
+        <v>0.007232640092706113</v>
       </c>
       <c r="C25" t="n">
+        <v>0.004556168732215964</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.003576046962064411</v>
+      </c>
+      <c r="E25" t="n">
         <v>0.2288103047304828</v>
       </c>
-      <c r="D25" t="n">
+      <c r="F25" t="n">
         <v>0.0113311104787564</v>
       </c>
-      <c r="E25" t="n">
+      <c r="G25" t="n">
+        <v>0.002810559911499391</v>
+      </c>
+      <c r="H25" t="n">
         <v>0.1330630664437363</v>
       </c>
-      <c r="F25" t="n">
+      <c r="I25" t="n">
         <v>0.3830434986033608</v>
       </c>
-      <c r="G25" t="n">
+      <c r="J25" t="n">
         <v>0.4379239125040536</v>
       </c>
     </row>
@@ -1067,21 +1298,30 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.212535502847336</v>
+        <v>0.009066654713756232</v>
       </c>
       <c r="C26" t="n">
+        <v>0.006691611377560857</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.006182383005475539</v>
+      </c>
+      <c r="E26" t="n">
         <v>0.3061139916364429</v>
       </c>
-      <c r="D26" t="n">
+      <c r="F26" t="n">
         <v>0.01518937977458646</v>
       </c>
-      <c r="E26" t="n">
+      <c r="G26" t="n">
+        <v>0.005656559037128603</v>
+      </c>
+      <c r="H26" t="n">
         <v>0.1236482354395601</v>
       </c>
-      <c r="F26" t="n">
+      <c r="I26" t="n">
         <v>0.5435414116365747</v>
       </c>
-      <c r="G26" t="n">
+      <c r="J26" t="n">
         <v>0.6086005322782936</v>
       </c>
     </row>
@@ -1092,21 +1332,30 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.1764250174245969</v>
+        <v>0.007494801021133443</v>
       </c>
       <c r="C27" t="n">
+        <v>0.005030660090075821</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.004297382221991953</v>
+      </c>
+      <c r="E27" t="n">
         <v>0.2541196998187805</v>
       </c>
-      <c r="D27" t="n">
+      <c r="F27" t="n">
         <v>0.01221458249795926</v>
       </c>
-      <c r="E27" t="n">
+      <c r="G27" t="n">
+        <v>0.005588299784399712</v>
+      </c>
+      <c r="H27" t="n">
         <v>0.1226277551044361</v>
       </c>
-      <c r="F27" t="n">
+      <c r="I27" t="n">
         <v>0.4473582352546316</v>
       </c>
-      <c r="G27" t="n">
+      <c r="J27" t="n">
         <v>0.4888205014789123</v>
       </c>
     </row>
@@ -1117,21 +1366,30 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.2093176821651463</v>
+        <v>0.008976964720763557</v>
       </c>
       <c r="C28" t="n">
+        <v>0.006574876335923587</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.006030513026017032</v>
+      </c>
+      <c r="E28" t="n">
         <v>0.3014954352915672</v>
       </c>
-      <c r="D28" t="n">
+      <c r="F28" t="n">
         <v>0.01452470582250177</v>
       </c>
-      <c r="E28" t="n">
+      <c r="G28" t="n">
+        <v>0.005130528286225509</v>
+      </c>
+      <c r="H28" t="n">
         <v>0.1194296820038135</v>
       </c>
-      <c r="F28" t="n">
+      <c r="I28" t="n">
         <v>0.5380487723240551</v>
       </c>
-      <c r="G28" t="n">
+      <c r="J28" t="n">
         <v>0.5987931802282037</v>
       </c>
     </row>
@@ -1142,21 +1400,30 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.17863376681167</v>
+        <v>0.007580794437988916</v>
       </c>
       <c r="C29" t="n">
+        <v>0.005124150576556056</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.004418361440659265</v>
+      </c>
+      <c r="E29" t="n">
         <v>0.2572758750122056</v>
       </c>
-      <c r="D29" t="n">
+      <c r="F29" t="n">
         <v>0.01247693938442809</v>
       </c>
-      <c r="E29" t="n">
+      <c r="G29" t="n">
+        <v>0.005995837971417423</v>
+      </c>
+      <c r="H29" t="n">
         <v>0.1236963263892</v>
       </c>
-      <c r="F29" t="n">
+      <c r="I29" t="n">
         <v>0.4532637956100669</v>
       </c>
-      <c r="G29" t="n">
+      <c r="J29" t="n">
         <v>0.4951528146379342</v>
       </c>
     </row>
@@ -1167,21 +1434,30 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.1834859983358927</v>
+        <v>0.007356619676443914</v>
       </c>
       <c r="C30" t="n">
+        <v>0.005014207609025327</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.004255370284274993</v>
+      </c>
+      <c r="E30" t="n">
         <v>0.2641647091160827</v>
       </c>
-      <c r="D30" t="n">
+      <c r="F30" t="n">
         <v>0.01318191958664414</v>
       </c>
-      <c r="E30" t="n">
+      <c r="G30" t="n">
+        <v>0.003781681943601781</v>
+      </c>
+      <c r="H30" t="n">
         <v>0.129863314993275</v>
       </c>
-      <c r="F30" t="n">
+      <c r="I30" t="n">
         <v>0.4502705273495035</v>
       </c>
-      <c r="G30" t="n">
+      <c r="J30" t="n">
         <v>0.5212485979616395</v>
       </c>
     </row>
@@ -1192,21 +1468,30 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.1571050544306945</v>
+        <v>0.006248800583661181</v>
       </c>
       <c r="C31" t="n">
+        <v>0.003913476260874994</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.003054812223113419</v>
+      </c>
+      <c r="E31" t="n">
         <v>0.226170251822342</v>
       </c>
-      <c r="D31" t="n">
+      <c r="F31" t="n">
         <v>0.01066598117504436</v>
       </c>
-      <c r="E31" t="n">
+      <c r="G31" t="n">
+        <v>0.002917633297931239</v>
+      </c>
+      <c r="H31" t="n">
         <v>0.1244190096543001</v>
       </c>
-      <c r="F31" t="n">
+      <c r="I31" t="n">
         <v>0.3871086188970695</v>
       </c>
-      <c r="G31" t="n">
+      <c r="J31" t="n">
         <v>0.4314124039331906</v>
       </c>
     </row>
@@ -1217,21 +1502,30 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.179397843026922</v>
+        <v>0.007256352243478374</v>
       </c>
       <c r="C32" t="n">
+        <v>0.004877061785380903</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.004063814981930763</v>
+      </c>
+      <c r="E32" t="n">
         <v>0.2582943095061376</v>
       </c>
-      <c r="D32" t="n">
+      <c r="F32" t="n">
         <v>0.01290855245898198</v>
       </c>
-      <c r="E32" t="n">
+      <c r="G32" t="n">
+        <v>0.003056229348808458</v>
+      </c>
+      <c r="H32" t="n">
         <v>0.1309382059445011</v>
       </c>
-      <c r="F32" t="n">
+      <c r="I32" t="n">
         <v>0.4371945612868097</v>
       </c>
-      <c r="G32" t="n">
+      <c r="J32" t="n">
         <v>0.508522282967191</v>
       </c>
     </row>
@@ -1242,21 +1536,30 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.1525201027955786</v>
+        <v>0.006096123198365482</v>
       </c>
       <c r="C33" t="n">
+        <v>0.003754189684709533</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.002878096873367812</v>
+      </c>
+      <c r="E33" t="n">
         <v>0.2195597271000847</v>
       </c>
-      <c r="D33" t="n">
+      <c r="F33" t="n">
         <v>0.01052988316386006</v>
       </c>
-      <c r="E33" t="n">
+      <c r="G33" t="n">
+        <v>0.002603960820847316</v>
+      </c>
+      <c r="H33" t="n">
         <v>0.128466209797355</v>
       </c>
-      <c r="F33" t="n">
+      <c r="I33" t="n">
         <v>0.3711855392649482</v>
       </c>
-      <c r="G33" t="n">
+      <c r="J33" t="n">
         <v>0.4156835882566379</v>
       </c>
     </row>
@@ -1267,21 +1570,30 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.2183437431886787</v>
+        <v>0.007847517827452719</v>
       </c>
       <c r="C34" t="n">
+        <v>0.005838990819378964</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.005380616214774134</v>
+      </c>
+      <c r="E34" t="n">
         <v>0.3144860329840703</v>
       </c>
-      <c r="D34" t="n">
+      <c r="F34" t="n">
         <v>0.01586697527357359</v>
       </c>
-      <c r="E34" t="n">
+      <c r="G34" t="n">
+        <v>0.005496344511155615</v>
+      </c>
+      <c r="H34" t="n">
         <v>0.1260550062309409</v>
       </c>
-      <c r="F34" t="n">
+      <c r="I34" t="n">
         <v>0.5556335079279879</v>
       </c>
-      <c r="G34" t="n">
+      <c r="J34" t="n">
         <v>0.6290898562805615</v>
       </c>
     </row>
@@ -1292,21 +1604,30 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.1862243568217817</v>
+        <v>0.006868013454898184</v>
       </c>
       <c r="C35" t="n">
+        <v>0.004747704161729377</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.00417908646944658</v>
+      </c>
+      <c r="E35" t="n">
         <v>0.268246952991507</v>
       </c>
-      <c r="D35" t="n">
+      <c r="F35" t="n">
         <v>0.01351005738177668</v>
       </c>
-      <c r="E35" t="n">
+      <c r="G35" t="n">
+        <v>0.006836269503404424</v>
+      </c>
+      <c r="H35" t="n">
         <v>0.1286220392116503</v>
       </c>
-      <c r="F35" t="n">
+      <c r="I35" t="n">
         <v>0.469444885808481</v>
       </c>
-      <c r="G35" t="n">
+      <c r="J35" t="n">
         <v>0.5194915519739046</v>
       </c>
     </row>
@@ -1317,21 +1638,30 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.2099229839341403</v>
+        <v>0.007582726832618118</v>
       </c>
       <c r="C36" t="n">
+        <v>0.005532554875060244</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.005019461465359231</v>
+      </c>
+      <c r="E36" t="n">
         <v>0.3023932030168321</v>
       </c>
-      <c r="D36" t="n">
+      <c r="F36" t="n">
         <v>0.0152465988571365</v>
       </c>
-      <c r="E36" t="n">
+      <c r="G36" t="n">
+        <v>0.005518166051649107</v>
+      </c>
+      <c r="H36" t="n">
         <v>0.1269623071159753</v>
       </c>
-      <c r="F36" t="n">
+      <c r="I36" t="n">
         <v>0.5302909665980746</v>
       </c>
-      <c r="G36" t="n">
+      <c r="J36" t="n">
         <v>0.6031504042422905</v>
       </c>
     </row>
@@ -1342,21 +1672,30 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.1907922691979433</v>
+        <v>0.007004079354472999</v>
       </c>
       <c r="C37" t="n">
+        <v>0.004896498748180307</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.004345258718978713</v>
+      </c>
+      <c r="E37" t="n">
         <v>0.2747788699687923</v>
       </c>
-      <c r="D37" t="n">
+      <c r="F37" t="n">
         <v>0.01379527335796418</v>
       </c>
-      <c r="E37" t="n">
+      <c r="G37" t="n">
+        <v>0.007164442981635558</v>
+      </c>
+      <c r="H37" t="n">
         <v>0.127512683054028</v>
       </c>
-      <c r="F37" t="n">
+      <c r="I37" t="n">
         <v>0.4833493825964172</v>
       </c>
-      <c r="G37" t="n">
+      <c r="J37" t="n">
         <v>0.5341683609211683</v>
       </c>
     </row>
@@ -1367,21 +1706,30 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.192023571346495</v>
+        <v>0.007562876382774937</v>
       </c>
       <c r="C38" t="n">
+        <v>0.005280052486482614</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.00457177537947798</v>
+      </c>
+      <c r="E38" t="n">
         <v>0.2765279245471765</v>
       </c>
-      <c r="D38" t="n">
+      <c r="F38" t="n">
         <v>0.0136318292613619</v>
       </c>
-      <c r="E38" t="n">
+      <c r="G38" t="n">
+        <v>0.002894491029822271</v>
+      </c>
+      <c r="H38" t="n">
         <v>0.1260088267770148</v>
       </c>
-      <c r="F38" t="n">
+      <c r="I38" t="n">
         <v>0.4796840810042629</v>
       </c>
-      <c r="G38" t="n">
+      <c r="J38" t="n">
         <v>0.5472735227691808</v>
       </c>
     </row>
@@ -1392,21 +1740,30 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.1727148355913672</v>
+        <v>0.00667466990266271</v>
       </c>
       <c r="C39" t="n">
+        <v>0.0044065752821592</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.003648699943497079</v>
+      </c>
+      <c r="E39" t="n">
         <v>0.2485951048069859</v>
       </c>
-      <c r="D39" t="n">
+      <c r="F39" t="n">
         <v>0.01193687848534092</v>
       </c>
-      <c r="E39" t="n">
+      <c r="G39" t="n">
+        <v>0.004406860222294219</v>
+      </c>
+      <c r="H39" t="n">
         <v>0.1238769680236924</v>
       </c>
-      <c r="F39" t="n">
+      <c r="I39" t="n">
         <v>0.4334751788306641</v>
       </c>
-      <c r="G39" t="n">
+      <c r="J39" t="n">
         <v>0.4791860285957047</v>
       </c>
     </row>
@@ -1417,21 +1774,30 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.1953787441682979</v>
+        <v>0.007632379821909612</v>
       </c>
       <c r="C40" t="n">
+        <v>0.005372882116869902</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.004679476359102669</v>
+      </c>
+      <c r="E40" t="n">
         <v>0.2813384696438941</v>
       </c>
-      <c r="D40" t="n">
+      <c r="F40" t="n">
         <v>0.01412384439663287</v>
       </c>
-      <c r="E40" t="n">
+      <c r="G40" t="n">
+        <v>0.003139176747071001</v>
+      </c>
+      <c r="H40" t="n">
         <v>0.1285739341599941</v>
       </c>
-      <c r="F40" t="n">
+      <c r="I40" t="n">
         <v>0.486418269406426</v>
       </c>
-      <c r="G40" t="n">
+      <c r="J40" t="n">
         <v>0.5578299309728705</v>
       </c>
     </row>
@@ -1442,21 +1808,30 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.1683899904559086</v>
+        <v>0.006551684168406867</v>
       </c>
       <c r="C41" t="n">
+        <v>0.00426420404842502</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.003472349918576316</v>
+      </c>
+      <c r="E41" t="n">
         <v>0.2423846872729665</v>
       </c>
-      <c r="D41" t="n">
+      <c r="F41" t="n">
         <v>0.0115616367765186</v>
       </c>
-      <c r="E41" t="n">
+      <c r="G41" t="n">
+        <v>0.003912484663575528</v>
+      </c>
+      <c r="H41" t="n">
         <v>0.1236131866094931</v>
       </c>
-      <c r="F41" t="n">
+      <c r="I41" t="n">
         <v>0.4211407039374992</v>
       </c>
-      <c r="G41" t="n">
+      <c r="J41" t="n">
         <v>0.4658127501610339</v>
       </c>
     </row>
@@ -1467,21 +1842,30 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.2314625445513873</v>
+        <v>0.00826369073122956</v>
       </c>
       <c r="C42" t="n">
+        <v>0.006375077806801487</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.00614210460104269</v>
+      </c>
+      <c r="E42" t="n">
         <v>0.3331517495080442</v>
       </c>
-      <c r="D42" t="n">
+      <c r="F42" t="n">
         <v>0.01678666810572753</v>
       </c>
-      <c r="E42" t="n">
+      <c r="G42" t="n">
+        <v>0.008747931088492717</v>
+      </c>
+      <c r="H42" t="n">
         <v>0.1244160279166226</v>
       </c>
-      <c r="F42" t="n">
+      <c r="I42" t="n">
         <v>0.5981045801620152</v>
       </c>
-      <c r="G42" t="n">
+      <c r="J42" t="n">
         <v>0.6666366589168998</v>
       </c>
     </row>
@@ -1492,21 +1876,30 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.1918956959975996</v>
+        <v>0.006937908852255941</v>
       </c>
       <c r="C43" t="n">
+        <v>0.004861404835373084</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.004308365239629935</v>
+      </c>
+      <c r="E43" t="n">
         <v>0.2763146565069083</v>
       </c>
-      <c r="D43" t="n">
+      <c r="F43" t="n">
         <v>0.01278761023554117</v>
       </c>
-      <c r="E43" t="n">
+      <c r="G43" t="n">
+        <v>0.006935834364679067</v>
+      </c>
+      <c r="H43" t="n">
         <v>0.1147670936662415</v>
       </c>
-      <c r="F43" t="n">
+      <c r="I43" t="n">
         <v>0.5003432226239096</v>
       </c>
-      <c r="G43" t="n">
+      <c r="J43" t="n">
         <v>0.5366027339557026</v>
       </c>
     </row>
@@ -1517,21 +1910,30 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.2339714347351005</v>
+        <v>0.00836872874071392</v>
       </c>
       <c r="C44" t="n">
+        <v>0.006504464623928063</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.006330396109457286</v>
+      </c>
+      <c r="E44" t="n">
         <v>0.3368600483830249</v>
       </c>
-      <c r="D44" t="n">
+      <c r="F44" t="n">
         <v>0.01694778106507748</v>
       </c>
-      <c r="E44" t="n">
+      <c r="G44" t="n">
+        <v>0.009277518770060337</v>
+      </c>
+      <c r="H44" t="n">
         <v>0.1236521420543296</v>
       </c>
-      <c r="F44" t="n">
+      <c r="I44" t="n">
         <v>0.606482623975393</v>
       </c>
-      <c r="G44" t="n">
+      <c r="J44" t="n">
         <v>0.6740248009670742</v>
       </c>
     </row>
@@ -1542,21 +1944,30 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.1963085408288961</v>
+        <v>0.0070948713090124</v>
       </c>
       <c r="C45" t="n">
+        <v>0.005036369215028862</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.004537850370715181</v>
+      </c>
+      <c r="E45" t="n">
         <v>0.2826979014998394</v>
       </c>
-      <c r="D45" t="n">
+      <c r="F45" t="n">
         <v>0.01337086329517205</v>
       </c>
-      <c r="E45" t="n">
+      <c r="G45" t="n">
+        <v>0.00801285210215146</v>
+      </c>
+      <c r="H45" t="n">
         <v>0.1171378270520285</v>
       </c>
-      <c r="F45" t="n">
+      <c r="I45" t="n">
         <v>0.5117463208452449</v>
       </c>
-      <c r="G45" t="n">
+      <c r="J45" t="n">
         <v>0.5491760954778077</v>
       </c>
     </row>
@@ -1567,21 +1978,30 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.2051323967361419</v>
+        <v>0.007717671250130857</v>
       </c>
       <c r="C46" t="n">
+        <v>0.005592051873185065</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.005093677973007158</v>
+      </c>
+      <c r="E46" t="n">
         <v>0.2954827941030577</v>
       </c>
-      <c r="D46" t="n">
+      <c r="F46" t="n">
         <v>0.01437030680455617</v>
       </c>
-      <c r="E46" t="n">
+      <c r="G46" t="n">
+        <v>0.005532309650961178</v>
+      </c>
+      <c r="H46" t="n">
         <v>0.1213322249670894</v>
       </c>
-      <c r="F46" t="n">
+      <c r="I46" t="n">
         <v>0.524027953286105</v>
       </c>
-      <c r="G46" t="n">
+      <c r="J46" t="n">
         <v>0.58588288229119</v>
       </c>
     </row>
@@ -1592,21 +2012,30 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.1776199912792987</v>
+        <v>0.006574271394817817</v>
       </c>
       <c r="C47" t="n">
+        <v>0.004432059496680291</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.003808987551583259</v>
+      </c>
+      <c r="E47" t="n">
         <v>0.2558060384537857</v>
       </c>
-      <c r="D47" t="n">
+      <c r="F47" t="n">
         <v>0.0125626730786941</v>
       </c>
-      <c r="E47" t="n">
+      <c r="G47" t="n">
+        <v>0.005768766735005136</v>
+      </c>
+      <c r="H47" t="n">
         <v>0.1264918573268463</v>
       </c>
-      <c r="F47" t="n">
+      <c r="I47" t="n">
         <v>0.4437094665070302</v>
       </c>
-      <c r="G47" t="n">
+      <c r="J47" t="n">
         <v>0.4956940505294836</v>
       </c>
     </row>
@@ -1617,21 +2046,30 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.2138316047183999</v>
+        <v>0.007897466454061475</v>
       </c>
       <c r="C48" t="n">
+        <v>0.005843558526638881</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.005419937765964188</v>
+      </c>
+      <c r="E48" t="n">
         <v>0.3080044116849983</v>
       </c>
-      <c r="D48" t="n">
+      <c r="F48" t="n">
         <v>0.01522302947130069</v>
       </c>
-      <c r="E48" t="n">
+      <c r="G48" t="n">
+        <v>0.00599760405161546</v>
+      </c>
+      <c r="H48" t="n">
         <v>0.1229039181501574</v>
       </c>
-      <c r="F48" t="n">
+      <c r="I48" t="n">
         <v>0.5469823969335205</v>
       </c>
-      <c r="G48" t="n">
+      <c r="J48" t="n">
         <v>0.6134918820354418</v>
       </c>
     </row>
@@ -1642,21 +2080,30 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.178835094305252</v>
+        <v>0.006507077943525411</v>
       </c>
       <c r="C49" t="n">
+        <v>0.004397221998847755</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.00377157708652045</v>
+      </c>
+      <c r="E49" t="n">
         <v>0.2575858540232248</v>
       </c>
-      <c r="D49" t="n">
+      <c r="F49" t="n">
         <v>0.01231533406395668</v>
       </c>
-      <c r="E49" t="n">
+      <c r="G49" t="n">
+        <v>0.005633787244288565</v>
+      </c>
+      <c r="H49" t="n">
         <v>0.1217237360775313</v>
       </c>
-      <c r="F49" t="n">
+      <c r="I49" t="n">
         <v>0.4522465633547929</v>
       </c>
-      <c r="G49" t="n">
+      <c r="J49" t="n">
         <v>0.4992361861849257</v>
       </c>
     </row>
@@ -1667,21 +2114,30 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.2096574435185962</v>
+        <v>0.007863034276754966</v>
       </c>
       <c r="C50" t="n">
+        <v>0.005783102835262788</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.005335054986094638</v>
+      </c>
+      <c r="E50" t="n">
         <v>0.3020317142542901</v>
       </c>
-      <c r="D50" t="n">
+      <c r="F50" t="n">
         <v>0.01484518121727406</v>
       </c>
-      <c r="E50" t="n">
+      <c r="G50" t="n">
+        <v>0.004929984920625477</v>
+      </c>
+      <c r="H50" t="n">
         <v>0.1228266357467474</v>
       </c>
-      <c r="F50" t="n">
+      <c r="I50" t="n">
         <v>0.5331226396481293</v>
       </c>
-      <c r="G50" t="n">
+      <c r="J50" t="n">
         <v>0.6025748806787109</v>
       </c>
     </row>
@@ -1692,21 +2148,30 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.202261521417963</v>
+        <v>0.00752608289677562</v>
       </c>
       <c r="C51" t="n">
+        <v>0.005462072918412005</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.005114679388540377</v>
+      </c>
+      <c r="E51" t="n">
         <v>0.2913494986098453</v>
       </c>
-      <c r="D51" t="n">
+      <c r="F51" t="n">
         <v>0.01470000532845868</v>
       </c>
-      <c r="E51" t="n">
+      <c r="G51" t="n">
+        <v>0.01061809208529648</v>
+      </c>
+      <c r="H51" t="n">
         <v>0.1262339302300412</v>
       </c>
-      <c r="F51" t="n">
+      <c r="I51" t="n">
         <v>0.5190818176101127</v>
       </c>
-      <c r="G51" t="n">
+      <c r="J51" t="n">
         <v>0.5684538277366918</v>
       </c>
     </row>
@@ -1717,21 +2182,30 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.2172403766315923</v>
+        <v>0.008547808532776646</v>
       </c>
       <c r="C52" t="n">
+        <v>0.006365542216629994</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.005893631802469733</v>
+      </c>
+      <c r="E52" t="n">
         <v>0.3128843351814119</v>
       </c>
-      <c r="D52" t="n">
+      <c r="F52" t="n">
         <v>0.01591124570943957</v>
       </c>
-      <c r="E52" t="n">
+      <c r="G52" t="n">
+        <v>0.005770251795851536</v>
+      </c>
+      <c r="H52" t="n">
         <v>0.1272676465638826</v>
       </c>
-      <c r="F52" t="n">
+      <c r="I52" t="n">
         <v>0.5524295567745254</v>
       </c>
-      <c r="G52" t="n">
+      <c r="J52" t="n">
         <v>0.6244849440057852</v>
       </c>
     </row>
@@ -1742,21 +2216,30 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.1695397691998372</v>
+        <v>0.006806902837087269</v>
       </c>
       <c r="C53" t="n">
+        <v>0.004453581401047434</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.003648677668908566</v>
+      </c>
+      <c r="E53" t="n">
         <v>0.2441058525446645</v>
       </c>
-      <c r="D53" t="n">
+      <c r="F53" t="n">
         <v>0.01064115221664759</v>
       </c>
-      <c r="E53" t="n">
+      <c r="G53" t="n">
+        <v>0.003785584679996369</v>
+      </c>
+      <c r="H53" t="n">
         <v>0.1095531254244994</v>
       </c>
-      <c r="F53" t="n">
+      <c r="I53" t="n">
         <v>0.4372289679724848</v>
       </c>
-      <c r="G53" t="n">
+      <c r="J53" t="n">
         <v>0.4706079681771776</v>
       </c>
     </row>
@@ -1767,21 +2250,30 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.2213573771168423</v>
+        <v>0.008626719395224219</v>
       </c>
       <c r="C54" t="n">
+        <v>0.006479696739199757</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.006026459312608434</v>
+      </c>
+      <c r="E54" t="n">
         <v>0.31884245052578</v>
       </c>
-      <c r="D54" t="n">
+      <c r="F54" t="n">
         <v>0.0165366438427741</v>
       </c>
-      <c r="E54" t="n">
+      <c r="G54" t="n">
+        <v>0.005583008400228941</v>
+      </c>
+      <c r="H54" t="n">
         <v>0.1300470229506906</v>
       </c>
-      <c r="F54" t="n">
+      <c r="I54" t="n">
         <v>0.5610752353307057</v>
       </c>
-      <c r="G54" t="n">
+      <c r="J54" t="n">
         <v>0.6378427789687088</v>
       </c>
     </row>
@@ -1792,21 +2284,30 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.1671942020279725</v>
+        <v>0.006753053768726354</v>
       </c>
       <c r="C55" t="n">
+        <v>0.004387689324604164</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.003575254452984187</v>
+      </c>
+      <c r="E55" t="n">
         <v>0.2406680075190758</v>
       </c>
-      <c r="D55" t="n">
+      <c r="F55" t="n">
         <v>0.01042577518702069</v>
       </c>
-      <c r="E55" t="n">
+      <c r="G55" t="n">
+        <v>0.003694846206470743</v>
+      </c>
+      <c r="H55" t="n">
         <v>0.1090991216640434</v>
       </c>
-      <c r="F55" t="n">
+      <c r="I55" t="n">
         <v>0.4317064527771038</v>
       </c>
-      <c r="G55" t="n">
+      <c r="J55" t="n">
         <v>0.4625210541820744</v>
       </c>
     </row>
@@ -1817,21 +2318,30 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.2136144794408231</v>
+        <v>0.00891533985719703</v>
       </c>
       <c r="C56" t="n">
+        <v>0.006613680466964322</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.006120792532250954</v>
+      </c>
+      <c r="E56" t="n">
         <v>0.3075816706867506</v>
       </c>
-      <c r="D56" t="n">
+      <c r="F56" t="n">
         <v>0.01439174925538036</v>
       </c>
-      <c r="E56" t="n">
+      <c r="G56" t="n">
+        <v>0.004861612619090567</v>
+      </c>
+      <c r="H56" t="n">
         <v>0.1151850791905087</v>
       </c>
-      <c r="F56" t="n">
+      <c r="I56" t="n">
         <v>0.5530170149226139</v>
       </c>
-      <c r="G56" t="n">
+      <c r="J56" t="n">
         <v>0.6138401248019558</v>
       </c>
     </row>
@@ -1842,21 +2352,30 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.1717198187987923</v>
+        <v>0.007120820272283584</v>
       </c>
       <c r="C57" t="n">
+        <v>0.004697828078577773</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.00389476031709715</v>
+      </c>
+      <c r="E57" t="n">
         <v>0.2472813412914531</v>
       </c>
-      <c r="D57" t="n">
+      <c r="F57" t="n">
         <v>0.01090610195081238</v>
       </c>
-      <c r="E57" t="n">
+      <c r="G57" t="n">
+        <v>0.004122882193756804</v>
+      </c>
+      <c r="H57" t="n">
         <v>0.1107921349153157</v>
       </c>
-      <c r="F57" t="n">
+      <c r="I57" t="n">
         <v>0.442768397630447</v>
       </c>
-      <c r="G57" t="n">
+      <c r="J57" t="n">
         <v>0.4769839458794934</v>
       </c>
     </row>
@@ -1867,21 +2386,30 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.2165994475231497</v>
+        <v>0.008967112817091219</v>
       </c>
       <c r="C58" t="n">
+        <v>0.006684350981120694</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.00620346707786178</v>
+      </c>
+      <c r="E58" t="n">
         <v>0.3118771295516334</v>
       </c>
-      <c r="D58" t="n">
+      <c r="F58" t="n">
         <v>0.01517814207640768</v>
       </c>
-      <c r="E58" t="n">
+      <c r="G58" t="n">
+        <v>0.00550995433703646</v>
+      </c>
+      <c r="H58" t="n">
         <v>0.120796191257762</v>
       </c>
-      <c r="F58" t="n">
+      <c r="I58" t="n">
         <v>0.5551370228216943</v>
       </c>
-      <c r="G58" t="n">
+      <c r="J58" t="n">
         <v>0.6240194659254978</v>
       </c>
     </row>
@@ -1892,21 +2420,30 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.1745802376155472</v>
+        <v>0.007248179754153035</v>
       </c>
       <c r="C59" t="n">
+        <v>0.004823347564296571</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.00403340170280886</v>
+      </c>
+      <c r="E59" t="n">
         <v>0.2513534854633606</v>
       </c>
-      <c r="D59" t="n">
+      <c r="F59" t="n">
         <v>0.01104937795437904</v>
       </c>
-      <c r="E59" t="n">
+      <c r="G59" t="n">
+        <v>0.004315380467315962</v>
+      </c>
+      <c r="H59" t="n">
         <v>0.1101232755592692</v>
       </c>
-      <c r="F59" t="n">
+      <c r="I59" t="n">
         <v>0.4508300890592217</v>
       </c>
-      <c r="G59" t="n">
+      <c r="J59" t="n">
         <v>0.4867571139063996</v>
       </c>
     </row>
@@ -1917,21 +2454,30 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.2314224016012557</v>
+        <v>0.009485827463931723</v>
       </c>
       <c r="C60" t="n">
+        <v>0.007339817030528651</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.00713131403476465</v>
+      </c>
+      <c r="E60" t="n">
         <v>0.3333585627487622</v>
       </c>
-      <c r="D60" t="n">
+      <c r="F60" t="n">
         <v>0.01653789380134733</v>
       </c>
-      <c r="E60" t="n">
+      <c r="G60" t="n">
+        <v>0.008658949213229628</v>
+      </c>
+      <c r="H60" t="n">
         <v>0.1214414247338196</v>
       </c>
-      <c r="F60" t="n">
+      <c r="I60" t="n">
         <v>0.6013285140825689</v>
       </c>
-      <c r="G60" t="n">
+      <c r="J60" t="n">
         <v>0.6663130677707202</v>
       </c>
     </row>
@@ -1942,21 +2488,30 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.1983738227913925</v>
+        <v>0.008197497032157179</v>
       </c>
       <c r="C61" t="n">
+        <v>0.005861946818186317</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.005323889110002594</v>
+      </c>
+      <c r="E61" t="n">
         <v>0.2857246175325008</v>
       </c>
-      <c r="D61" t="n">
+      <c r="F61" t="n">
         <v>0.0131905710572662</v>
       </c>
-      <c r="E61" t="n">
+      <c r="G61" t="n">
+        <v>0.007588595209720587</v>
+      </c>
+      <c r="H61" t="n">
         <v>0.1136205992153412</v>
       </c>
-      <c r="F61" t="n">
+      <c r="I61" t="n">
         <v>0.5180996746042166</v>
       </c>
-      <c r="G61" t="n">
+      <c r="J61" t="n">
         <v>0.5587418739759767</v>
       </c>
     </row>
@@ -1967,21 +2522,30 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.2292603425325533</v>
+        <v>0.0093250565428312</v>
       </c>
       <c r="C62" t="n">
+        <v>0.007167609002413355</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.006896670300955492</v>
+      </c>
+      <c r="E62" t="n">
         <v>0.3302319537956788</v>
       </c>
-      <c r="D62" t="n">
+      <c r="F62" t="n">
         <v>0.01632489892419905</v>
       </c>
-      <c r="E62" t="n">
+      <c r="G62" t="n">
+        <v>0.007486255406269568</v>
+      </c>
+      <c r="H62" t="n">
         <v>0.1211952625195951</v>
       </c>
-      <c r="F62" t="n">
+      <c r="I62" t="n">
         <v>0.5947969173922354</v>
       </c>
-      <c r="G62" t="n">
+      <c r="J62" t="n">
         <v>0.6600598767063736</v>
       </c>
     </row>
@@ -1992,21 +2556,30 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.1934793174431852</v>
+        <v>0.007981415356531676</v>
       </c>
       <c r="C63" t="n">
+        <v>0.005631344246028453</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.005046329842092971</v>
+      </c>
+      <c r="E63" t="n">
         <v>0.2785922491985056</v>
       </c>
-      <c r="D63" t="n">
+      <c r="F63" t="n">
         <v>0.01278816025255028</v>
       </c>
-      <c r="E63" t="n">
+      <c r="G63" t="n">
+        <v>0.007086224275212159</v>
+      </c>
+      <c r="H63" t="n">
         <v>0.1135445814480387</v>
       </c>
-      <c r="F63" t="n">
+      <c r="I63" t="n">
         <v>0.5040815391247656</v>
       </c>
-      <c r="G63" t="n">
+      <c r="J63" t="n">
         <v>0.5434726068728011</v>
       </c>
     </row>
@@ -2017,21 +2590,30 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.2244126445063646</v>
+        <v>0.008448728872325848</v>
       </c>
       <c r="C64" t="n">
+        <v>0.00643634955366719</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.006174160534255983</v>
+      </c>
+      <c r="E64" t="n">
         <v>0.323193771030748</v>
       </c>
-      <c r="D64" t="n">
+      <c r="F64" t="n">
         <v>0.01610715961163545</v>
       </c>
-      <c r="E64" t="n">
+      <c r="G64" t="n">
+        <v>0.00841583673472854</v>
+      </c>
+      <c r="H64" t="n">
         <v>0.1231649857849427</v>
       </c>
-      <c r="F64" t="n">
+      <c r="I64" t="n">
         <v>0.5777622194990721</v>
       </c>
-      <c r="G64" t="n">
+      <c r="J64" t="n">
         <v>0.6460582763440706</v>
       </c>
     </row>
@@ -2042,21 +2624,30 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.1925153935610321</v>
+        <v>0.007227627952703827</v>
       </c>
       <c r="C65" t="n">
+        <v>0.005081631524275888</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.004529485612264172</v>
+      </c>
+      <c r="E65" t="n">
         <v>0.2772274024370305</v>
       </c>
-      <c r="D65" t="n">
+      <c r="F65" t="n">
         <v>0.01261675440052305</v>
       </c>
-      <c r="E65" t="n">
+      <c r="G65" t="n">
+        <v>0.007020361340799477</v>
+      </c>
+      <c r="H65" t="n">
         <v>0.1126276099426575</v>
       </c>
-      <c r="F65" t="n">
+      <c r="I65" t="n">
         <v>0.5002363437629563</v>
       </c>
-      <c r="G65" t="n">
+      <c r="J65" t="n">
         <v>0.5424567819047382</v>
       </c>
     </row>
@@ -2067,21 +2658,30 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.2305176185622087</v>
+        <v>0.008578118990436848</v>
       </c>
       <c r="C66" t="n">
+        <v>0.006621004028482609</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.006415313125324838</v>
+      </c>
+      <c r="E66" t="n">
         <v>0.332075039169702</v>
       </c>
-      <c r="D66" t="n">
+      <c r="F66" t="n">
         <v>0.01672991855189202</v>
       </c>
-      <c r="E66" t="n">
+      <c r="G66" t="n">
+        <v>0.008475453461030463</v>
+      </c>
+      <c r="H66" t="n">
         <v>0.1240253842545109</v>
       </c>
-      <c r="F66" t="n">
+      <c r="I66" t="n">
         <v>0.5945204656539936</v>
       </c>
-      <c r="G66" t="n">
+      <c r="J66" t="n">
         <v>0.6650912522519814</v>
       </c>
     </row>
@@ -2092,21 +2692,30 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.1941288359241782</v>
+        <v>0.007261264260530796</v>
       </c>
       <c r="C67" t="n">
+        <v>0.005134896360777016</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.00461859544499028</v>
+      </c>
+      <c r="E67" t="n">
         <v>0.2795509775860208</v>
       </c>
-      <c r="D67" t="n">
+      <c r="F67" t="n">
         <v>0.01269748560102469</v>
       </c>
-      <c r="E67" t="n">
+      <c r="G67" t="n">
+        <v>0.007575181026972662</v>
+      </c>
+      <c r="H67" t="n">
         <v>0.1120989456068729</v>
       </c>
-      <c r="F67" t="n">
+      <c r="I67" t="n">
         <v>0.5056506165123473</v>
       </c>
-      <c r="G67" t="n">
+      <c r="J67" t="n">
         <v>0.5472140494203661</v>
       </c>
     </row>
@@ -2117,21 +2726,30 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.2032242985951661</v>
+        <v>0.007317860077287968</v>
       </c>
       <c r="C68" t="n">
+        <v>0.005257496578180702</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0.004694058740406115</v>
+      </c>
+      <c r="E68" t="n">
         <v>0.2926667186422951</v>
       </c>
-      <c r="D68" t="n">
+      <c r="F68" t="n">
         <v>0.01441853496050546</v>
       </c>
-      <c r="E68" t="n">
+      <c r="G68" t="n">
+        <v>0.004301002067661788</v>
+      </c>
+      <c r="H68" t="n">
         <v>0.1241186321359398</v>
       </c>
-      <c r="F68" t="n">
+      <c r="I68" t="n">
         <v>0.5141936104415352</v>
       </c>
-      <c r="G68" t="n">
+      <c r="J68" t="n">
         <v>0.5816286332967258</v>
       </c>
     </row>
@@ -2142,21 +2760,30 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.1692029096775303</v>
+        <v>0.006093551272569017</v>
       </c>
       <c r="C69" t="n">
+        <v>0.003977182797829109</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0.003236463657029839</v>
+      </c>
+      <c r="E69" t="n">
         <v>0.2436905108806245</v>
       </c>
-      <c r="D69" t="n">
+      <c r="F69" t="n">
         <v>0.0109579309417184</v>
       </c>
-      <c r="E69" t="n">
+      <c r="G69" t="n">
+        <v>0.00326345410688235</v>
+      </c>
+      <c r="H69" t="n">
         <v>0.1140467102121938</v>
       </c>
-      <c r="F69" t="n">
+      <c r="I69" t="n">
         <v>0.4313064715245136</v>
       </c>
-      <c r="G69" t="n">
+      <c r="J69" t="n">
         <v>0.4701168432380169</v>
       </c>
     </row>
@@ -2167,21 +2794,30 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.204266446999383</v>
+        <v>0.007315177609986461</v>
       </c>
       <c r="C70" t="n">
+        <v>0.005281673771342648</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.004750664774391046</v>
+      </c>
+      <c r="E70" t="n">
         <v>0.2942390716222217</v>
       </c>
-      <c r="D70" t="n">
+      <c r="F70" t="n">
         <v>0.0147278913102918</v>
       </c>
-      <c r="E70" t="n">
+      <c r="G70" t="n">
+        <v>0.004691009698598479</v>
+      </c>
+      <c r="H70" t="n">
         <v>0.1264587630808758</v>
       </c>
-      <c r="F70" t="n">
+      <c r="I70" t="n">
         <v>0.5147304950870626</v>
       </c>
-      <c r="G70" t="n">
+      <c r="J70" t="n">
         <v>0.5852091644881955</v>
       </c>
     </row>
@@ -2192,21 +2828,30 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.1694501292872228</v>
+        <v>0.006071438473616384</v>
       </c>
       <c r="C71" t="n">
+        <v>0.003962381843061601</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.00321941125560668</v>
+      </c>
+      <c r="E71" t="n">
         <v>0.2439468810365941</v>
       </c>
-      <c r="D71" t="n">
+      <c r="F71" t="n">
         <v>0.01091174083793528</v>
       </c>
-      <c r="E71" t="n">
+      <c r="G71" t="n">
+        <v>0.00328843514049247</v>
+      </c>
+      <c r="H71" t="n">
         <v>0.1135420743133984</v>
       </c>
-      <c r="F71" t="n">
+      <c r="I71" t="n">
         <v>0.4313729446774021</v>
       </c>
-      <c r="G71" t="n">
+      <c r="J71" t="n">
         <v>0.47195664575702</v>
       </c>
     </row>
@@ -2217,21 +2862,30 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.2489998200825805</v>
+        <v>0.009361920093784613</v>
       </c>
       <c r="C72" t="n">
+        <v>0.007560651851252987</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.007737172553994796</v>
+      </c>
+      <c r="E72" t="n">
         <v>0.3587029766292162</v>
       </c>
-      <c r="D72" t="n">
+      <c r="F72" t="n">
         <v>0.01733076433606613</v>
       </c>
-      <c r="E72" t="n">
+      <c r="G72" t="n">
+        <v>0.01151223818795395</v>
+      </c>
+      <c r="H72" t="n">
         <v>0.1162651845138728</v>
       </c>
-      <c r="F72" t="n">
+      <c r="I72" t="n">
         <v>0.6567050083170408</v>
       </c>
-      <c r="G72" t="n">
+      <c r="J72" t="n">
         <v>0.7214243308097866</v>
       </c>
     </row>
@@ -2242,21 +2896,30 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.2049385811075486</v>
+        <v>0.007750712996969742</v>
       </c>
       <c r="C73" t="n">
+        <v>0.005684794463477289</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.005420624556326627</v>
+      </c>
+      <c r="E73" t="n">
         <v>0.2952052512983099</v>
       </c>
-      <c r="D73" t="n">
+      <c r="F73" t="n">
         <v>0.01432208746832835</v>
       </c>
-      <c r="E73" t="n">
+      <c r="G73" t="n">
+        <v>0.01244307627622545</v>
+      </c>
+      <c r="H73" t="n">
         <v>0.1195407042543856</v>
       </c>
-      <c r="F73" t="n">
+      <c r="I73" t="n">
         <v>0.536015610267085</v>
       </c>
-      <c r="G73" t="n">
+      <c r="J73" t="n">
         <v>0.5742375441407984</v>
       </c>
     </row>
@@ -2267,21 +2930,30 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.2514329030853613</v>
+        <v>0.009517469565303601</v>
       </c>
       <c r="C74" t="n">
+        <v>0.007719934466100909</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0.007913729629813951</v>
+      </c>
+      <c r="E74" t="n">
         <v>0.362201738082901</v>
       </c>
-      <c r="D74" t="n">
+      <c r="F74" t="n">
         <v>0.01661809628253856</v>
       </c>
-      <c r="E74" t="n">
+      <c r="G74" t="n">
+        <v>0.01031171210856489</v>
+      </c>
+      <c r="H74" t="n">
         <v>0.1092114173325418</v>
       </c>
-      <c r="F74" t="n">
+      <c r="I74" t="n">
         <v>0.6716635014282291</v>
       </c>
-      <c r="G74" t="n">
+      <c r="J74" t="n">
         <v>0.728253970444286</v>
       </c>
     </row>
@@ -2292,21 +2964,30 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.205793175762353</v>
+        <v>0.007825252418793418</v>
       </c>
       <c r="C75" t="n">
+        <v>0.005745772928550403</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0.005466717818460507</v>
+      </c>
+      <c r="E75" t="n">
         <v>0.296475770844133</v>
       </c>
-      <c r="D75" t="n">
+      <c r="F75" t="n">
         <v>0.0142144341103887</v>
       </c>
-      <c r="E75" t="n">
+      <c r="G75" t="n">
+        <v>0.01207560589443755</v>
+      </c>
+      <c r="H75" t="n">
         <v>0.1176690854107109</v>
       </c>
-      <c r="F75" t="n">
+      <c r="I75" t="n">
         <v>0.5399108281946081</v>
       </c>
-      <c r="G75" t="n">
+      <c r="J75" t="n">
         <v>0.5773594739180695</v>
       </c>
     </row>
@@ -2317,21 +2998,30 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.2136696059639608</v>
+        <v>0.008119021765466555</v>
       </c>
       <c r="C76" t="n">
+        <v>0.00600300905960356</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0.005521932534498927</v>
+      </c>
+      <c r="E76" t="n">
         <v>0.3075532034140523</v>
       </c>
-      <c r="D76" t="n">
+      <c r="F76" t="n">
         <v>0.01488648481925353</v>
       </c>
-      <c r="E76" t="n">
+      <c r="G76" t="n">
+        <v>0.005673539376447406</v>
+      </c>
+      <c r="H76" t="n">
         <v>0.1204521913439236</v>
       </c>
-      <c r="F76" t="n">
+      <c r="I76" t="n">
         <v>0.5480137663707879</v>
       </c>
-      <c r="G76" t="n">
+      <c r="J76" t="n">
         <v>0.6140353633671475</v>
       </c>
     </row>
@@ -2342,21 +3032,30 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.182957499923032</v>
+        <v>0.006915592441882048</v>
       </c>
       <c r="C77" t="n">
+        <v>0.004710650693984511</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0.00401819117273242</v>
+      </c>
+      <c r="E77" t="n">
         <v>0.2634048560151814</v>
       </c>
-      <c r="D77" t="n">
+      <c r="F77" t="n">
         <v>0.01210500000717565</v>
       </c>
-      <c r="E77" t="n">
+      <c r="G77" t="n">
+        <v>0.004901085185381464</v>
+      </c>
+      <c r="H77" t="n">
         <v>0.115464942369786</v>
       </c>
-      <c r="F77" t="n">
+      <c r="I77" t="n">
         <v>0.4690326851280835</v>
       </c>
-      <c r="G77" t="n">
+      <c r="J77" t="n">
         <v>0.5134645260978715</v>
       </c>
     </row>
@@ -2367,21 +3066,30 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.2236735087842915</v>
+        <v>0.008541255333797047</v>
       </c>
       <c r="C78" t="n">
+        <v>0.006486462172037498</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0.006160321584472095</v>
+      </c>
+      <c r="E78" t="n">
         <v>0.3220572119142466</v>
       </c>
-      <c r="D78" t="n">
+      <c r="F78" t="n">
         <v>0.01501723191603782</v>
       </c>
-      <c r="E78" t="n">
+      <c r="G78" t="n">
+        <v>0.006854333916835635</v>
+      </c>
+      <c r="H78" t="n">
         <v>0.1137933749699135</v>
       </c>
-      <c r="F78" t="n">
+      <c r="I78" t="n">
         <v>0.584004521469514</v>
       </c>
-      <c r="G78" t="n">
+      <c r="J78" t="n">
         <v>0.6445773422660266</v>
       </c>
     </row>
@@ -2392,21 +3100,30 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.1938248159173478</v>
+        <v>0.007282394221947247</v>
       </c>
       <c r="C79" t="n">
+        <v>0.005116822937055401</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.00451478319759455</v>
+      </c>
+      <c r="E79" t="n">
         <v>0.2790531159203484</v>
       </c>
-      <c r="D79" t="n">
+      <c r="F79" t="n">
         <v>0.01297233269713188</v>
       </c>
-      <c r="E79" t="n">
+      <c r="G79" t="n">
+        <v>0.006311623819257596</v>
+      </c>
+      <c r="H79" t="n">
         <v>0.1156318880305692</v>
       </c>
-      <c r="F79" t="n">
+      <c r="I79" t="n">
         <v>0.5008233861869779</v>
       </c>
-      <c r="G79" t="n">
+      <c r="J79" t="n">
         <v>0.5467362230830153</v>
       </c>
     </row>
@@ -2417,21 +3134,30 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.216902730502693</v>
+        <v>0.007482224832436913</v>
       </c>
       <c r="C80" t="n">
+        <v>0.005532837994218785</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0.005059686228222247</v>
+      </c>
+      <c r="E80" t="n">
         <v>0.3120990243464739</v>
       </c>
-      <c r="D80" t="n">
+      <c r="F80" t="n">
         <v>0.01658640024427636</v>
       </c>
-      <c r="E80" t="n">
+      <c r="G80" t="n">
+        <v>0.006210599621626118</v>
+      </c>
+      <c r="H80" t="n">
         <v>0.1353082786641611</v>
       </c>
-      <c r="F80" t="n">
+      <c r="I80" t="n">
         <v>0.5414721651945074</v>
       </c>
-      <c r="G80" t="n">
+      <c r="J80" t="n">
         <v>0.625305170453197</v>
       </c>
     </row>
@@ -2442,21 +3168,30 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.168908339188731</v>
+        <v>0.006060637139106459</v>
       </c>
       <c r="C81" t="n">
+        <v>0.003979573930338306</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0.003322973798354564</v>
+      </c>
+      <c r="E81" t="n">
         <v>0.2431545107302528</v>
       </c>
-      <c r="D81" t="n">
+      <c r="F81" t="n">
         <v>0.01167643596701807</v>
       </c>
-      <c r="E81" t="n">
+      <c r="G81" t="n">
+        <v>0.004618608752215418</v>
+      </c>
+      <c r="H81" t="n">
         <v>0.1248171542082588</v>
       </c>
-      <c r="F81" t="n">
+      <c r="I81" t="n">
         <v>0.420272207134426</v>
       </c>
-      <c r="G81" t="n">
+      <c r="J81" t="n">
         <v>0.4696401645124627</v>
       </c>
     </row>
@@ -2467,21 +3202,30 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.2029781178734204</v>
+        <v>0.007727293462595921</v>
       </c>
       <c r="C82" t="n">
+        <v>0.00556236515622225</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.004967779470164415</v>
+      </c>
+      <c r="E82" t="n">
         <v>0.2922773038327657</v>
       </c>
-      <c r="D82" t="n">
+      <c r="F82" t="n">
         <v>0.01319748803564807</v>
       </c>
-      <c r="E82" t="n">
+      <c r="G82" t="n">
+        <v>0.003142276018925362</v>
+      </c>
+      <c r="H82" t="n">
         <v>0.1115391176296462</v>
       </c>
-      <c r="F82" t="n">
+      <c r="I82" t="n">
         <v>0.5236061904455463</v>
       </c>
-      <c r="G82" t="n">
+      <c r="J82" t="n">
         <v>0.5830237029307115</v>
       </c>
     </row>
@@ -2492,21 +3236,30 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.1798343846550068</v>
+        <v>0.006833791486230323</v>
       </c>
       <c r="C83" t="n">
+        <v>0.004611569507002288</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0.003886248796901554</v>
+      </c>
+      <c r="E83" t="n">
         <v>0.2589205023139682</v>
       </c>
-      <c r="D83" t="n">
+      <c r="F83" t="n">
         <v>0.01085145099895932</v>
       </c>
-      <c r="E83" t="n">
+      <c r="G83" t="n">
+        <v>0.003945316693237234</v>
+      </c>
+      <c r="H83" t="n">
         <v>0.1032870702713524</v>
       </c>
-      <c r="F83" t="n">
+      <c r="I83" t="n">
         <v>0.4703863208128744</v>
       </c>
-      <c r="G83" t="n">
+      <c r="J83" t="n">
         <v>0.5054458512053621</v>
       </c>
     </row>
@@ -2517,21 +3270,30 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.1976953372206688</v>
+        <v>0.007496754111896646</v>
       </c>
       <c r="C84" t="n">
+        <v>0.005325759018421581</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0.004703990053473036</v>
+      </c>
+      <c r="E84" t="n">
         <v>0.2846727878196351</v>
       </c>
-      <c r="D84" t="n">
+      <c r="F84" t="n">
         <v>0.01334923416736708</v>
       </c>
-      <c r="E84" t="n">
+      <c r="G84" t="n">
+        <v>0.003637320933481595</v>
+      </c>
+      <c r="H84" t="n">
         <v>0.1176119142571492</v>
       </c>
-      <c r="F84" t="n">
+      <c r="I84" t="n">
         <v>0.5020249197241431</v>
       </c>
-      <c r="G84" t="n">
+      <c r="J84" t="n">
         <v>0.5669136801325032</v>
       </c>
     </row>
@@ -2542,21 +3304,30 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.1727796549594338</v>
+        <v>0.006632744664568133</v>
       </c>
       <c r="C85" t="n">
+        <v>0.004374959391400647</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0.003588093679985635</v>
+      </c>
+      <c r="E85" t="n">
         <v>0.2486740474733193</v>
       </c>
-      <c r="D85" t="n">
+      <c r="F85" t="n">
         <v>0.01033578457449792</v>
       </c>
-      <c r="E85" t="n">
+      <c r="G85" t="n">
+        <v>0.003212196042443065</v>
+      </c>
+      <c r="H85" t="n">
         <v>0.1032385919978487</v>
       </c>
-      <c r="F85" t="n">
+      <c r="I85" t="n">
         <v>0.44973640288866</v>
       </c>
-      <c r="G85" t="n">
+      <c r="J85" t="n">
         <v>0.4837932765809999</v>
       </c>
     </row>
@@ -2567,21 +3338,30 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.2079476706688584</v>
+        <v>0.008310303720439907</v>
       </c>
       <c r="C86" t="n">
+        <v>0.006050798792032853</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0.005466695850964662</v>
+      </c>
+      <c r="E86" t="n">
         <v>0.2994204453057663</v>
       </c>
-      <c r="D86" t="n">
+      <c r="F86" t="n">
         <v>0.01423035696195668</v>
       </c>
-      <c r="E86" t="n">
+      <c r="G86" t="n">
+        <v>0.005062319145832996</v>
+      </c>
+      <c r="H86" t="n">
         <v>0.1181739377757453</v>
       </c>
-      <c r="F86" t="n">
+      <c r="I86" t="n">
         <v>0.5333714268382356</v>
       </c>
-      <c r="G86" t="n">
+      <c r="J86" t="n">
         <v>0.5967108433440163</v>
       </c>
     </row>
@@ -2592,21 +3372,30 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1869631893168628</v>
+        <v>0.007412738621709655</v>
       </c>
       <c r="C87" t="n">
+        <v>0.005086605862907996</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0.004320271308676339</v>
+      </c>
+      <c r="E87" t="n">
         <v>0.2690462145388953</v>
       </c>
-      <c r="D87" t="n">
+      <c r="F87" t="n">
         <v>0.01156578049481163</v>
       </c>
-      <c r="E87" t="n">
+      <c r="G87" t="n">
+        <v>0.004169048015564303</v>
+      </c>
+      <c r="H87" t="n">
         <v>0.106083258292596</v>
       </c>
-      <c r="F87" t="n">
+      <c r="I87" t="n">
         <v>0.4887545408311644</v>
       </c>
-      <c r="G87" t="n">
+      <c r="J87" t="n">
         <v>0.5271222233979582</v>
       </c>
     </row>
@@ -2617,21 +3406,30 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.2177499041777636</v>
+        <v>0.008860744700533161</v>
       </c>
       <c r="C88" t="n">
+        <v>0.006658965177386253</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0.006315585408014424</v>
+      </c>
+      <c r="E88" t="n">
         <v>0.3135685079604867</v>
       </c>
-      <c r="D88" t="n">
+      <c r="F88" t="n">
         <v>0.01602015029797256</v>
       </c>
-      <c r="E88" t="n">
+      <c r="G88" t="n">
+        <v>0.008355541827185516</v>
+      </c>
+      <c r="H88" t="n">
         <v>0.128236921795885</v>
       </c>
-      <c r="F88" t="n">
+      <c r="I88" t="n">
         <v>0.5526076221276424</v>
       </c>
-      <c r="G88" t="n">
+      <c r="J88" t="n">
         <v>0.627896613549452</v>
       </c>
     </row>
@@ -2642,21 +3440,30 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.1830367207704417</v>
+        <v>0.007732521862391008</v>
       </c>
       <c r="C89" t="n">
+        <v>0.005311771088613373</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0.00466317745769089</v>
+      </c>
+      <c r="E89" t="n">
         <v>0.2636345436605838</v>
       </c>
-      <c r="D89" t="n">
+      <c r="F89" t="n">
         <v>0.01212226763148952</v>
       </c>
-      <c r="E89" t="n">
+      <c r="G89" t="n">
+        <v>0.006632290787882547</v>
+      </c>
+      <c r="H89" t="n">
         <v>0.1156255515128127</v>
       </c>
-      <c r="F89" t="n">
+      <c r="I89" t="n">
         <v>0.4664462882143972</v>
       </c>
-      <c r="G89" t="n">
+      <c r="J89" t="n">
         <v>0.5164941608233885</v>
       </c>
     </row>
@@ -2667,21 +3474,30 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.207815690366772</v>
+        <v>0.008374514348112204</v>
       </c>
       <c r="C90" t="n">
+        <v>0.006090753817015875</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0.005471788911413704</v>
+      </c>
+      <c r="E90" t="n">
         <v>0.2992246583121921</v>
       </c>
-      <c r="D90" t="n">
+      <c r="F90" t="n">
         <v>0.01451213972703367</v>
       </c>
-      <c r="E90" t="n">
+      <c r="G90" t="n">
+        <v>0.003572570945257205</v>
+      </c>
+      <c r="H90" t="n">
         <v>0.1214709691700149</v>
       </c>
-      <c r="F90" t="n">
+      <c r="I90" t="n">
         <v>0.5289163426845562</v>
       </c>
-      <c r="G90" t="n">
+      <c r="J90" t="n">
         <v>0.5972635022112321</v>
       </c>
     </row>
@@ -2692,21 +3508,30 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.1704496778845069</v>
+        <v>0.006924893560951662</v>
       </c>
       <c r="C91" t="n">
+        <v>0.00454772062478472</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0.003759134729436284</v>
+      </c>
+      <c r="E91" t="n">
         <v>0.2454631603532006</v>
       </c>
-      <c r="D91" t="n">
+      <c r="F91" t="n">
         <v>0.01109275497828015</v>
       </c>
-      <c r="E91" t="n">
+      <c r="G91" t="n">
+        <v>0.004350125493488509</v>
+      </c>
+      <c r="H91" t="n">
         <v>0.1142739611528542</v>
       </c>
-      <c r="F91" t="n">
+      <c r="I91" t="n">
         <v>0.4376990825818318</v>
       </c>
-      <c r="G91" t="n">
+      <c r="J91" t="n">
         <v>0.4709190492599948</v>
       </c>
     </row>
@@ -2717,21 +3542,30 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.2015139993134965</v>
+        <v>0.008143633029701723</v>
       </c>
       <c r="C92" t="n">
+        <v>0.005819848881082356</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0.005139969992081844</v>
+      </c>
+      <c r="E92" t="n">
         <v>0.2900982556392546</v>
       </c>
-      <c r="D92" t="n">
+      <c r="F92" t="n">
         <v>0.01373633573399875</v>
       </c>
-      <c r="E92" t="n">
+      <c r="G92" t="n">
+        <v>0.003451248042550532</v>
+      </c>
+      <c r="H92" t="n">
         <v>0.1185143963679092</v>
       </c>
-      <c r="F92" t="n">
+      <c r="I92" t="n">
         <v>0.5141610306345479</v>
       </c>
-      <c r="G92" t="n">
+      <c r="J92" t="n">
         <v>0.5768506332537132</v>
       </c>
     </row>
@@ -2742,21 +3576,30 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.1714880026792206</v>
+        <v>0.006980571858482171</v>
       </c>
       <c r="C93" t="n">
+        <v>0.004603899213927553</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0.003831307386579222</v>
+      </c>
+      <c r="E93" t="n">
         <v>0.2469023387819733</v>
       </c>
-      <c r="D93" t="n">
+      <c r="F93" t="n">
         <v>0.0112132388243184</v>
       </c>
-      <c r="E93" t="n">
+      <c r="G93" t="n">
+        <v>0.004586547373106695</v>
+      </c>
+      <c r="H93" t="n">
         <v>0.1149754244660972</v>
       </c>
-      <c r="F93" t="n">
+      <c r="I93" t="n">
         <v>0.4398446883017233</v>
       </c>
-      <c r="G93" t="n">
+      <c r="J93" t="n">
         <v>0.4742723346651463</v>
       </c>
     </row>
@@ -2767,21 +3610,30 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.2081218136257766</v>
+        <v>0.007151316118722072</v>
       </c>
       <c r="C94" t="n">
+        <v>0.00522343082357488</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0.004771184542493839</v>
+      </c>
+      <c r="E94" t="n">
         <v>0.2996955574431795</v>
       </c>
-      <c r="D94" t="n">
+      <c r="F94" t="n">
         <v>0.01520952205325705</v>
       </c>
-      <c r="E94" t="n">
+      <c r="G94" t="n">
+        <v>0.005239647033376329</v>
+      </c>
+      <c r="H94" t="n">
         <v>0.1283178132539637</v>
       </c>
-      <c r="F94" t="n">
+      <c r="I94" t="n">
         <v>0.5238124071380009</v>
       </c>
-      <c r="G94" t="n">
+      <c r="J94" t="n">
         <v>0.5969674162907299</v>
       </c>
     </row>
@@ -2792,21 +3644,30 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.1762636907994085</v>
+        <v>0.006077214182684828</v>
       </c>
       <c r="C95" t="n">
+        <v>0.004064724491328476</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0.003423154990094223</v>
+      </c>
+      <c r="E95" t="n">
         <v>0.2538500510821917</v>
       </c>
-      <c r="D95" t="n">
+      <c r="F95" t="n">
         <v>0.01223258752081313</v>
       </c>
-      <c r="E95" t="n">
+      <c r="G95" t="n">
+        <v>0.004932121488960246</v>
+      </c>
+      <c r="H95" t="n">
         <v>0.1233718528854208</v>
       </c>
-      <c r="F95" t="n">
+      <c r="I95" t="n">
         <v>0.4447873648889497</v>
       </c>
-      <c r="G95" t="n">
+      <c r="J95" t="n">
         <v>0.4896730793002917</v>
       </c>
     </row>
@@ -2817,21 +3678,30 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.2052752102603077</v>
+        <v>0.007122808486141482</v>
       </c>
       <c r="C96" t="n">
+        <v>0.005174602155114322</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0.004727545281284593</v>
+      </c>
+      <c r="E96" t="n">
         <v>0.2957369571460093</v>
       </c>
-      <c r="D96" t="n">
+      <c r="F96" t="n">
         <v>0.01477088378823554</v>
       </c>
-      <c r="E96" t="n">
+      <c r="G96" t="n">
+        <v>0.005902622703858181</v>
+      </c>
+      <c r="H96" t="n">
         <v>0.1255713082949788</v>
       </c>
-      <c r="F96" t="n">
+      <c r="I96" t="n">
         <v>0.5194228170979056</v>
       </c>
-      <c r="G96" t="n">
+      <c r="J96" t="n">
         <v>0.587183228233549</v>
       </c>
     </row>
@@ -2842,21 +3712,30 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.1773465219369219</v>
+        <v>0.006086714611150081</v>
       </c>
       <c r="C97" t="n">
+        <v>0.004083993169068166</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0.003455044663493903</v>
+      </c>
+      <c r="E97" t="n">
         <v>0.2554315012087314</v>
       </c>
-      <c r="D97" t="n">
+      <c r="F97" t="n">
         <v>0.01231635117866708</v>
       </c>
-      <c r="E97" t="n">
+      <c r="G97" t="n">
+        <v>0.005140344603891793</v>
+      </c>
+      <c r="H97" t="n">
         <v>0.1231839081924249</v>
       </c>
-      <c r="F97" t="n">
+      <c r="I97" t="n">
         <v>0.4483768473441985</v>
       </c>
-      <c r="G97" t="n">
+      <c r="J97" t="n">
         <v>0.49275627250698</v>
       </c>
     </row>
@@ -2867,21 +3746,30 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.2044401472453267</v>
+        <v>0.007355206615662204</v>
       </c>
       <c r="C98" t="n">
+        <v>0.00530726365757881</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0.004759297155012127</v>
+      </c>
+      <c r="E98" t="n">
         <v>0.2944615760214875</v>
       </c>
-      <c r="D98" t="n">
+      <c r="F98" t="n">
         <v>0.01462422671082877</v>
       </c>
-      <c r="E98" t="n">
+      <c r="G98" t="n">
+        <v>0.004483558557170285</v>
+      </c>
+      <c r="H98" t="n">
         <v>0.125338079845915</v>
       </c>
-      <c r="F98" t="n">
+      <c r="I98" t="n">
         <v>0.5152206379221079</v>
       </c>
-      <c r="G98" t="n">
+      <c r="J98" t="n">
         <v>0.5865966118823098</v>
       </c>
     </row>
@@ -2892,21 +3780,30 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.1798098620602101</v>
+        <v>0.006496335145476754</v>
       </c>
       <c r="C99" t="n">
+        <v>0.004400420360540669</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0.003777760547879593</v>
+      </c>
+      <c r="E99" t="n">
         <v>0.258854741842862</v>
       </c>
-      <c r="D99" t="n">
+      <c r="F99" t="n">
         <v>0.01207333495006717</v>
       </c>
-      <c r="E99" t="n">
+      <c r="G99" t="n">
+        <v>0.006057747438423491</v>
+      </c>
+      <c r="H99" t="n">
         <v>0.1175801551983707</v>
       </c>
-      <c r="F99" t="n">
+      <c r="I99" t="n">
         <v>0.462555637821173</v>
       </c>
-      <c r="G99" t="n">
+      <c r="J99" t="n">
         <v>0.4988302850264365</v>
       </c>
     </row>
@@ -2917,21 +3814,30 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.1932197585027936</v>
+        <v>0.007033062514173645</v>
       </c>
       <c r="C100" t="n">
+        <v>0.00492068818854686</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0.004274891249825489</v>
+      </c>
+      <c r="E100" t="n">
         <v>0.278272983996576</v>
       </c>
-      <c r="D100" t="n">
+      <c r="F100" t="n">
         <v>0.01358794561700337</v>
       </c>
-      <c r="E100" t="n">
+      <c r="G100" t="n">
+        <v>0.003795703349072984</v>
+      </c>
+      <c r="H100" t="n">
         <v>0.1238864723607382</v>
       </c>
-      <c r="F100" t="n">
+      <c r="I100" t="n">
         <v>0.4865661698452459</v>
       </c>
-      <c r="G100" t="n">
+      <c r="J100" t="n">
         <v>0.5494409227303361</v>
       </c>
     </row>
@@ -2942,21 +3848,30 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.1741427115656571</v>
+        <v>0.006376318938033967</v>
       </c>
       <c r="C101" t="n">
+        <v>0.004242115398048149</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0.003567559183909469</v>
+      </c>
+      <c r="E101" t="n">
         <v>0.2507526118376088</v>
       </c>
-      <c r="D101" t="n">
+      <c r="F101" t="n">
         <v>0.01166138854198479</v>
       </c>
-      <c r="E101" t="n">
+      <c r="G101" t="n">
+        <v>0.005212156070174176</v>
+      </c>
+      <c r="H101" t="n">
         <v>0.1179337175383456</v>
       </c>
-      <c r="F101" t="n">
+      <c r="I101" t="n">
         <v>0.445644130874921</v>
       </c>
-      <c r="G101" t="n">
+      <c r="J101" t="n">
         <v>0.4813832147627722</v>
       </c>
     </row>
@@ -2967,21 +3882,30 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.2089796881791465</v>
+        <v>0.008525861165371953</v>
       </c>
       <c r="C102" t="n">
+        <v>0.006228057520372983</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0.005625413409454035</v>
+      </c>
+      <c r="E102" t="n">
         <v>0.3008249278377101</v>
       </c>
-      <c r="D102" t="n">
+      <c r="F102" t="n">
         <v>0.01379526194026</v>
       </c>
-      <c r="E102" t="n">
+      <c r="G102" t="n">
+        <v>0.003699710477666059</v>
+      </c>
+      <c r="H102" t="n">
         <v>0.1131134974007003</v>
       </c>
-      <c r="F102" t="n">
+      <c r="I102" t="n">
         <v>0.5411580759936877</v>
       </c>
-      <c r="G102" t="n">
+      <c r="J102" t="n">
         <v>0.5999671682856248</v>
       </c>
     </row>
@@ -2992,21 +3916,30 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.1779257027029883</v>
+        <v>0.007283575012845086</v>
       </c>
       <c r="C103" t="n">
+        <v>0.004881251948536857</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0.004082673400943081</v>
+      </c>
+      <c r="E103" t="n">
         <v>0.2560724893630765</v>
       </c>
-      <c r="D103" t="n">
+      <c r="F103" t="n">
         <v>0.01126575622715563</v>
       </c>
-      <c r="E103" t="n">
+      <c r="G103" t="n">
+        <v>0.004188773086419675</v>
+      </c>
+      <c r="H103" t="n">
         <v>0.1100210201195701</v>
       </c>
-      <c r="F103" t="n">
+      <c r="I103" t="n">
         <v>0.4600566597828214</v>
       </c>
-      <c r="G103" t="n">
+      <c r="J103" t="n">
         <v>0.4976361962575837</v>
       </c>
     </row>
@@ -3017,21 +3950,30 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.2039517260539852</v>
+        <v>0.008365204314980654</v>
       </c>
       <c r="C104" t="n">
+        <v>0.006037111735264379</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.005398089932089038</v>
+      </c>
+      <c r="E104" t="n">
         <v>0.2935746702564633</v>
       </c>
-      <c r="D104" t="n">
+      <c r="F104" t="n">
         <v>0.01299976617755271</v>
       </c>
-      <c r="E104" t="n">
+      <c r="G104" t="n">
+        <v>0.003553871704108941</v>
+      </c>
+      <c r="H104" t="n">
         <v>0.1088293461994772</v>
       </c>
-      <c r="F104" t="n">
+      <c r="I104" t="n">
         <v>0.5312169137330149</v>
       </c>
-      <c r="G104" t="n">
+      <c r="J104" t="n">
         <v>0.5841594288807542</v>
       </c>
     </row>
@@ -3042,21 +3984,30 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.1776342432858412</v>
+        <v>0.007257724459895735</v>
       </c>
       <c r="C105" t="n">
+        <v>0.004858570217634571</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0.004057160518318965</v>
+      </c>
+      <c r="E105" t="n">
         <v>0.2557107765146632</v>
       </c>
-      <c r="D105" t="n">
+      <c r="F105" t="n">
         <v>0.01142636950681757</v>
       </c>
-      <c r="E105" t="n">
+      <c r="G105" t="n">
+        <v>0.004141623793213862</v>
+      </c>
+      <c r="H105" t="n">
         <v>0.1121105623655467</v>
       </c>
-      <c r="F105" t="n">
+      <c r="I105" t="n">
         <v>0.4575355926162823</v>
       </c>
-      <c r="G105" t="n">
+      <c r="J105" t="n">
         <v>0.4963410654943621</v>
       </c>
     </row>
@@ -3067,21 +4018,30 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.20089488220115</v>
+        <v>0.00776851382148951</v>
       </c>
       <c r="C106" t="n">
+        <v>0.005603564771985434</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0.005129312513075607</v>
+      </c>
+      <c r="E106" t="n">
         <v>0.2894657326637893</v>
       </c>
-      <c r="D106" t="n">
+      <c r="F106" t="n">
         <v>0.01504137299409666</v>
       </c>
-      <c r="E106" t="n">
+      <c r="G106" t="n">
+        <v>0.006121025415455896</v>
+      </c>
+      <c r="H106" t="n">
         <v>0.1336717928894148</v>
       </c>
-      <c r="F106" t="n">
+      <c r="I106" t="n">
         <v>0.4951678798533038</v>
       </c>
-      <c r="G106" t="n">
+      <c r="J106" t="n">
         <v>0.5771874661970106</v>
       </c>
     </row>
@@ -3092,21 +4052,30 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.1852108034871148</v>
+        <v>0.007125638344626567</v>
       </c>
       <c r="C107" t="n">
+        <v>0.004930898634910881</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0.004351537849822832</v>
+      </c>
+      <c r="E107" t="n">
         <v>0.2667774783649008</v>
       </c>
-      <c r="D107" t="n">
+      <c r="F107" t="n">
         <v>0.01183797370993214</v>
       </c>
-      <c r="E107" t="n">
+      <c r="G107" t="n">
+        <v>0.006199949822469107</v>
+      </c>
+      <c r="H107" t="n">
         <v>0.1096759117507966</v>
       </c>
-      <c r="F107" t="n">
+      <c r="I107" t="n">
         <v>0.4830054286100193</v>
       </c>
-      <c r="G107" t="n">
+      <c r="J107" t="n">
         <v>0.518813991216255</v>
       </c>
     </row>
@@ -3117,21 +4086,30 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.2065827782513615</v>
+        <v>0.00788923099593361</v>
       </c>
       <c r="C108" t="n">
+        <v>0.005776054559474609</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0.005356382287438284</v>
+      </c>
+      <c r="E108" t="n">
         <v>0.2976152993768065</v>
       </c>
-      <c r="D108" t="n">
+      <c r="F108" t="n">
         <v>0.01467035114391935</v>
       </c>
-      <c r="E108" t="n">
+      <c r="G108" t="n">
+        <v>0.006207874895193356</v>
+      </c>
+      <c r="H108" t="n">
         <v>0.1236841207036741</v>
       </c>
-      <c r="F108" t="n">
+      <c r="I108" t="n">
         <v>0.523671764449643</v>
       </c>
-      <c r="G108" t="n">
+      <c r="J108" t="n">
         <v>0.5930099181487326</v>
       </c>
     </row>
@@ -3142,21 +4120,30 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.1716747784873845</v>
+        <v>0.006785364517422766</v>
       </c>
       <c r="C109" t="n">
+        <v>0.004514249881140664</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0.00385856460422104</v>
+      </c>
+      <c r="E109" t="n">
         <v>0.2473758797681106</v>
       </c>
-      <c r="D109" t="n">
+      <c r="F109" t="n">
         <v>0.01121637475510564</v>
       </c>
-      <c r="E109" t="n">
+      <c r="G109" t="n">
+        <v>0.004937755785269454</v>
+      </c>
+      <c r="H109" t="n">
         <v>0.1145251571765398</v>
       </c>
-      <c r="F109" t="n">
+      <c r="I109" t="n">
         <v>0.4394629824865389</v>
       </c>
-      <c r="G109" t="n">
+      <c r="J109" t="n">
         <v>0.4767017252753354</v>
       </c>
     </row>
@@ -3167,21 +4154,30 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.2008623699789246</v>
+        <v>0.007846966197869173</v>
       </c>
       <c r="C110" t="n">
+        <v>0.00566307240042547</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0.005196268246986106</v>
+      </c>
+      <c r="E110" t="n">
         <v>0.2893738763353487</v>
       </c>
-      <c r="D110" t="n">
+      <c r="F110" t="n">
         <v>0.01500636117788512</v>
       </c>
-      <c r="E110" t="n">
+      <c r="G110" t="n">
+        <v>0.006274486780798834</v>
+      </c>
+      <c r="H110" t="n">
         <v>0.133705083827905</v>
       </c>
-      <c r="F110" t="n">
+      <c r="I110" t="n">
         <v>0.4950556464559735</v>
       </c>
-      <c r="G110" t="n">
+      <c r="J110" t="n">
         <v>0.5777670781182143</v>
       </c>
     </row>
@@ -3192,21 +4188,30 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.1892034109419499</v>
+        <v>0.007271886847709495</v>
       </c>
       <c r="C111" t="n">
+        <v>0.005093559709047713</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0.004560146685715967</v>
+      </c>
+      <c r="E111" t="n">
         <v>0.272440340968069</v>
       </c>
-      <c r="D111" t="n">
+      <c r="F111" t="n">
         <v>0.0119611181531596</v>
       </c>
-      <c r="E111" t="n">
+      <c r="G111" t="n">
+        <v>0.006875408543331441</v>
+      </c>
+      <c r="H111" t="n">
         <v>0.1080441296138627</v>
       </c>
-      <c r="F111" t="n">
+      <c r="I111" t="n">
         <v>0.4965194231342294</v>
       </c>
-      <c r="G111" t="n">
+      <c r="J111" t="n">
         <v>0.5312442324778349</v>
       </c>
     </row>
@@ -3217,21 +4222,30 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.2059617161251173</v>
+        <v>0.007867232771869237</v>
       </c>
       <c r="C112" t="n">
+        <v>0.005745744924586971</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0.005309587090872871</v>
+      </c>
+      <c r="E112" t="n">
         <v>0.2968046776930804</v>
       </c>
-      <c r="D112" t="n">
+      <c r="F112" t="n">
         <v>0.01458172985666335</v>
       </c>
-      <c r="E112" t="n">
+      <c r="G112" t="n">
+        <v>0.006015825400827664</v>
+      </c>
+      <c r="H112" t="n">
         <v>0.1232934676846422</v>
       </c>
-      <c r="F112" t="n">
+      <c r="I112" t="n">
         <v>0.5218722562959272</v>
       </c>
-      <c r="G112" t="n">
+      <c r="J112" t="n">
         <v>0.591933287218686</v>
       </c>
     </row>
@@ -3242,21 +4256,30 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.1711860140942047</v>
+        <v>0.00673828827073004</v>
       </c>
       <c r="C113" t="n">
+        <v>0.004475577840034291</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0.003824547839124124</v>
+      </c>
+      <c r="E113" t="n">
         <v>0.2466744354928498</v>
       </c>
-      <c r="D113" t="n">
+      <c r="F113" t="n">
         <v>0.01144533696073178</v>
       </c>
-      <c r="E113" t="n">
+      <c r="G113" t="n">
+        <v>0.004966049058638749</v>
+      </c>
+      <c r="H113" t="n">
         <v>0.1181519168281768</v>
       </c>
-      <c r="F113" t="n">
+      <c r="I113" t="n">
         <v>0.4343087498929015</v>
       </c>
-      <c r="G113" t="n">
+      <c r="J113" t="n">
         <v>0.4753016386759394</v>
       </c>
     </row>
@@ -3267,21 +4290,30 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.1974190589802542</v>
+        <v>0.008775549239816306</v>
       </c>
       <c r="C114" t="n">
+        <v>0.006252203311210293</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0.00558517665814869</v>
+      </c>
+      <c r="E114" t="n">
         <v>0.2844754664169857</v>
       </c>
-      <c r="D114" t="n">
+      <c r="F114" t="n">
         <v>0.01566263947061257</v>
       </c>
-      <c r="E114" t="n">
+      <c r="G114" t="n">
+        <v>0.004346758507844604</v>
+      </c>
+      <c r="H114" t="n">
         <v>0.1453482877216337</v>
       </c>
-      <c r="F114" t="n">
+      <c r="I114" t="n">
         <v>0.4748553481365727</v>
       </c>
-      <c r="G114" t="n">
+      <c r="J114" t="n">
         <v>0.5654456531205186</v>
       </c>
     </row>
@@ -3292,21 +4324,30 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.1573111508227613</v>
+        <v>0.007335028783801657</v>
       </c>
       <c r="C115" t="n">
+        <v>0.004651373175881315</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0.003774836061270101</v>
+      </c>
+      <c r="E115" t="n">
         <v>0.2266085950495241</v>
       </c>
-      <c r="D115" t="n">
+      <c r="F115" t="n">
         <v>0.009726730796116129</v>
       </c>
-      <c r="E115" t="n">
+      <c r="G115" t="n">
+        <v>0.003438680176931924</v>
+      </c>
+      <c r="H115" t="n">
         <v>0.1096147981879132</v>
       </c>
-      <c r="F115" t="n">
+      <c r="I115" t="n">
         <v>0.3988156565372212</v>
       </c>
-      <c r="G115" t="n">
+      <c r="J115" t="n">
         <v>0.4360140538780495</v>
       </c>
     </row>
@@ -3317,21 +4358,30 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.2065598828582323</v>
+        <v>0.009225602834137278</v>
       </c>
       <c r="C116" t="n">
+        <v>0.006737281147842313</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0.00620050488526443</v>
+      </c>
+      <c r="E116" t="n">
         <v>0.2977568028239566</v>
       </c>
-      <c r="D116" t="n">
+      <c r="F116" t="n">
         <v>0.01646234491666609</v>
       </c>
-      <c r="E116" t="n">
+      <c r="G116" t="n">
+        <v>0.005286722890192116</v>
+      </c>
+      <c r="H116" t="n">
         <v>0.1433840111153917</v>
       </c>
-      <c r="F116" t="n">
+      <c r="I116" t="n">
         <v>0.5052272433007947</v>
       </c>
-      <c r="G116" t="n">
+      <c r="J116" t="n">
         <v>0.5918907504582076</v>
       </c>
     </row>
@@ -3342,21 +4392,30 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.1679934222688014</v>
+        <v>0.007630524804169093</v>
       </c>
       <c r="C117" t="n">
+        <v>0.00500081103035032</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0.004170733468024358</v>
+      </c>
+      <c r="E117" t="n">
         <v>0.2419600893301629</v>
       </c>
-      <c r="D117" t="n">
+      <c r="F117" t="n">
         <v>0.01049367647178074</v>
       </c>
-      <c r="E117" t="n">
+      <c r="G117" t="n">
+        <v>0.004178515603783197</v>
+      </c>
+      <c r="H117" t="n">
         <v>0.1092345743410947</v>
       </c>
-      <c r="F117" t="n">
+      <c r="I117" t="n">
         <v>0.4313492516340939</v>
       </c>
-      <c r="G117" t="n">
+      <c r="J117" t="n">
         <v>0.4679888630709989</v>
       </c>
     </row>
@@ -3367,21 +4426,30 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.198095816962601</v>
+        <v>0.008409841612605306</v>
       </c>
       <c r="C118" t="n">
+        <v>0.006018387543064671</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0.005431584540169261</v>
+      </c>
+      <c r="E118" t="n">
         <v>0.2851616266116929</v>
       </c>
-      <c r="D118" t="n">
+      <c r="F118" t="n">
         <v>0.01264550945052318</v>
       </c>
-      <c r="E118" t="n">
+      <c r="G118" t="n">
+        <v>0.004677691038047582</v>
+      </c>
+      <c r="H118" t="n">
         <v>0.1097153437866304</v>
       </c>
-      <c r="F118" t="n">
+      <c r="I118" t="n">
         <v>0.5131664996238799</v>
       </c>
-      <c r="G118" t="n">
+      <c r="J118" t="n">
         <v>0.5667226607889528</v>
       </c>
     </row>
@@ -3392,21 +4460,30 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.1597131763359152</v>
+        <v>0.006690394830196923</v>
       </c>
       <c r="C119" t="n">
+        <v>0.004234296545689782</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0.003315123557855276</v>
+      </c>
+      <c r="E119" t="n">
         <v>0.2298791928272897</v>
       </c>
-      <c r="D119" t="n">
+      <c r="F119" t="n">
         <v>0.008838288502470416</v>
       </c>
-      <c r="E119" t="n">
+      <c r="G119" t="n">
+        <v>0.001904397768011703</v>
+      </c>
+      <c r="H119" t="n">
         <v>0.09554188467337478</v>
       </c>
-      <c r="F119" t="n">
+      <c r="I119" t="n">
         <v>0.416489300901951</v>
       </c>
-      <c r="G119" t="n">
+      <c r="J119" t="n">
         <v>0.4467868015242897</v>
       </c>
     </row>
@@ -3417,21 +4494,30 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.1829359002148268</v>
+        <v>0.00803616505554729</v>
       </c>
       <c r="C120" t="n">
+        <v>0.00550752213600043</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0.004771885128107081</v>
+      </c>
+      <c r="E120" t="n">
         <v>0.2635935013798111</v>
       </c>
-      <c r="D120" t="n">
+      <c r="F120" t="n">
         <v>0.01182892602359522</v>
       </c>
-      <c r="E120" t="n">
+      <c r="G120" t="n">
+        <v>0.003357468564474381</v>
+      </c>
+      <c r="H120" t="n">
         <v>0.1127642250509478</v>
       </c>
-      <c r="F120" t="n">
+      <c r="I120" t="n">
         <v>0.4649710396376155</v>
       </c>
-      <c r="G120" t="n">
+      <c r="J120" t="n">
         <v>0.5209793223664161</v>
       </c>
     </row>
@@ -3442,21 +4528,30 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.1522769252255721</v>
+        <v>0.006541478076229728</v>
       </c>
       <c r="C121" t="n">
+        <v>0.004036807378447232</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0.003091178862340368</v>
+      </c>
+      <c r="E121" t="n">
         <v>0.219293381577415</v>
       </c>
-      <c r="D121" t="n">
+      <c r="F121" t="n">
         <v>0.008625067982023565</v>
       </c>
-      <c r="E121" t="n">
+      <c r="G121" t="n">
+        <v>0.001616673207544682</v>
+      </c>
+      <c r="H121" t="n">
         <v>0.09903541686402963</v>
       </c>
-      <c r="F121" t="n">
+      <c r="I121" t="n">
         <v>0.3923609875213573</v>
       </c>
-      <c r="G121" t="n">
+      <c r="J121" t="n">
         <v>0.4228949134025182</v>
       </c>
     </row>
@@ -3467,21 +4562,30 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.2136653839606336</v>
+        <v>0.008721621121405941</v>
       </c>
       <c r="C122" t="n">
+        <v>0.006523620967395098</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.006269106014842799</v>
+      </c>
+      <c r="E122" t="n">
         <v>0.3078933480650645</v>
       </c>
-      <c r="D122" t="n">
+      <c r="F122" t="n">
         <v>0.01515536596126788</v>
       </c>
-      <c r="E122" t="n">
+      <c r="G122" t="n">
+        <v>0.009436800064958357</v>
+      </c>
+      <c r="H122" t="n">
         <v>0.1220355508959028</v>
       </c>
-      <c r="F122" t="n">
+      <c r="I122" t="n">
         <v>0.5487199579738571</v>
       </c>
-      <c r="G122" t="n">
+      <c r="J122" t="n">
         <v>0.6123040927850815</v>
       </c>
     </row>
@@ -3492,21 +4596,30 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.1533175413673585</v>
+        <v>0.00648420726245549</v>
       </c>
       <c r="C123" t="n">
+        <v>0.004053807846896905</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.003247639830737141</v>
+      </c>
+      <c r="E123" t="n">
         <v>0.2209016541922966</v>
       </c>
-      <c r="D123" t="n">
+      <c r="F123" t="n">
         <v>0.008922818453046181</v>
       </c>
-      <c r="E123" t="n">
+      <c r="G123" t="n">
+        <v>0.003104651767512235</v>
+      </c>
+      <c r="H123" t="n">
         <v>0.1016241751730903</v>
       </c>
-      <c r="F123" t="n">
+      <c r="I123" t="n">
         <v>0.3970957108111854</v>
       </c>
-      <c r="G123" t="n">
+      <c r="J123" t="n">
         <v>0.4217747465893332</v>
       </c>
     </row>
@@ -3517,21 +4630,30 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.2234537709075235</v>
+        <v>0.009165757714770028</v>
       </c>
       <c r="C124" t="n">
+        <v>0.007026830802352417</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.006949861609681651</v>
+      </c>
+      <c r="E124" t="n">
         <v>0.3219970998442295</v>
       </c>
-      <c r="D124" t="n">
+      <c r="F124" t="n">
         <v>0.01554824280595462</v>
       </c>
-      <c r="E124" t="n">
+      <c r="G124" t="n">
+        <v>0.01089987692871609</v>
+      </c>
+      <c r="H124" t="n">
         <v>0.1181037548714755</v>
       </c>
-      <c r="F124" t="n">
+      <c r="I124" t="n">
         <v>0.5810345487394867</v>
       </c>
-      <c r="G124" t="n">
+      <c r="J124" t="n">
         <v>0.6424644965078091</v>
       </c>
     </row>
@@ -3542,21 +4664,30 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.1714561091938501</v>
+        <v>0.007105236598632518</v>
       </c>
       <c r="C125" t="n">
+        <v>0.004712701041913741</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.003979181386386902</v>
+      </c>
+      <c r="E125" t="n">
         <v>0.2470166663696935</v>
       </c>
-      <c r="D125" t="n">
+      <c r="F125" t="n">
         <v>0.009970104999847814</v>
       </c>
-      <c r="E125" t="n">
+      <c r="G125" t="n">
+        <v>0.004230191127898567</v>
+      </c>
+      <c r="H125" t="n">
         <v>0.09903478397378768</v>
       </c>
-      <c r="F125" t="n">
+      <c r="I125" t="n">
         <v>0.4536354020723314</v>
       </c>
-      <c r="G125" t="n">
+      <c r="J125" t="n">
         <v>0.4766583605059554</v>
       </c>
     </row>
@@ -3567,21 +4698,30 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.2144910716825911</v>
+        <v>0.007831815755320153</v>
       </c>
       <c r="C126" t="n">
+        <v>0.005784602449028273</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.00528879746854677</v>
+      </c>
+      <c r="E126" t="n">
         <v>0.3089751961789997</v>
       </c>
-      <c r="D126" t="n">
+      <c r="F126" t="n">
         <v>0.01553134759613456</v>
       </c>
-      <c r="E126" t="n">
+      <c r="G126" t="n">
+        <v>0.004281174814516704</v>
+      </c>
+      <c r="H126" t="n">
         <v>0.1258073346514741</v>
       </c>
-      <c r="F126" t="n">
+      <c r="I126" t="n">
         <v>0.5446525422346403</v>
       </c>
-      <c r="G126" t="n">
+      <c r="J126" t="n">
         <v>0.6171682429485081</v>
       </c>
     </row>
@@ -3592,21 +4732,30 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.1429550246013129</v>
+        <v>0.006283739841061002</v>
       </c>
       <c r="C127" t="n">
+        <v>0.003718933615882197</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.002697841433154388</v>
+      </c>
+      <c r="E127" t="n">
         <v>0.2057195637625276</v>
       </c>
-      <c r="D127" t="n">
+      <c r="F127" t="n">
         <v>0.01000586093978007</v>
       </c>
-      <c r="E127" t="n">
+      <c r="G127" t="n">
+        <v>0.001566051724276981</v>
+      </c>
+      <c r="H127" t="n">
         <v>0.1355608921808412</v>
       </c>
-      <c r="F127" t="n">
+      <c r="I127" t="n">
         <v>0.3352921206764383</v>
       </c>
-      <c r="G127" t="n">
+      <c r="J127" t="n">
         <v>0.3875075318528641</v>
       </c>
     </row>
@@ -3617,21 +4766,30 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.1970510605520885</v>
+        <v>0.008381136307655336</v>
       </c>
       <c r="C128" t="n">
+        <v>0.005879406567096692</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.005054800192062594</v>
+      </c>
+      <c r="E128" t="n">
         <v>0.2838949235969464</v>
       </c>
-      <c r="D128" t="n">
+      <c r="F128" t="n">
         <v>0.01452031886637024</v>
       </c>
-      <c r="E128" t="n">
+      <c r="G128" t="n">
+        <v>0.002873424443738431</v>
+      </c>
+      <c r="H128" t="n">
         <v>0.1309769462084722</v>
       </c>
-      <c r="F128" t="n">
+      <c r="I128" t="n">
         <v>0.4905211826243687</v>
       </c>
-      <c r="G128" t="n">
+      <c r="J128" t="n">
         <v>0.5617468786499783</v>
       </c>
     </row>
@@ -3642,21 +4800,30 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.1674364773566707</v>
+        <v>0.007273926180305603</v>
       </c>
       <c r="C129" t="n">
+        <v>0.004721641113992426</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.003843277878323754</v>
+      </c>
+      <c r="E129" t="n">
         <v>0.2411615051141358</v>
       </c>
-      <c r="D129" t="n">
+      <c r="F129" t="n">
         <v>0.01169661874994026</v>
       </c>
-      <c r="E129" t="n">
+      <c r="G129" t="n">
+        <v>0.003900655598395762</v>
+      </c>
+      <c r="H129" t="n">
         <v>0.1264820817682941</v>
       </c>
-      <c r="F129" t="n">
+      <c r="I129" t="n">
         <v>0.4145566610396063</v>
       </c>
-      <c r="G129" t="n">
+      <c r="J129" t="n">
         <v>0.4638294980336164</v>
       </c>
     </row>
@@ -3667,21 +4834,30 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.1935586257499659</v>
+        <v>0.008434329357807427</v>
       </c>
       <c r="C130" t="n">
+        <v>0.005890273628774112</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.005076385471364516</v>
+      </c>
+      <c r="E130" t="n">
         <v>0.2788261314334571</v>
       </c>
-      <c r="D130" t="n">
+      <c r="F130" t="n">
         <v>0.0141169978535509</v>
       </c>
-      <c r="E130" t="n">
+      <c r="G130" t="n">
+        <v>0.002886064784164903</v>
+      </c>
+      <c r="H130" t="n">
         <v>0.1299646651741799</v>
       </c>
-      <c r="F130" t="n">
+      <c r="I130" t="n">
         <v>0.4800617327274269</v>
       </c>
-      <c r="G130" t="n">
+      <c r="J130" t="n">
         <v>0.5517725065579129</v>
       </c>
     </row>
@@ -3692,21 +4868,30 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.1715105039936793</v>
+        <v>0.007446438069495701</v>
       </c>
       <c r="C131" t="n">
+        <v>0.004899295052730374</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.004061947576313579</v>
+      </c>
+      <c r="E131" t="n">
         <v>0.2469933562431668</v>
       </c>
-      <c r="D131" t="n">
+      <c r="F131" t="n">
         <v>0.01228558305671909</v>
       </c>
-      <c r="E131" t="n">
+      <c r="G131" t="n">
+        <v>0.004812875973580303</v>
+      </c>
+      <c r="H131" t="n">
         <v>0.1298529671279539</v>
       </c>
-      <c r="F131" t="n">
+      <c r="I131" t="n">
         <v>0.4246095216989238</v>
       </c>
-      <c r="G131" t="n">
+      <c r="J131" t="n">
         <v>0.4749156184102663</v>
       </c>
     </row>
@@ -3717,21 +4902,30 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.1948371504044179</v>
+        <v>0.007467744409969876</v>
       </c>
       <c r="C132" t="n">
+        <v>0.00526502861136552</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0.004628974812338723</v>
+      </c>
+      <c r="E132" t="n">
         <v>0.2804740291690905</v>
       </c>
-      <c r="D132" t="n">
+      <c r="F132" t="n">
         <v>0.01261096891676533</v>
       </c>
-      <c r="E132" t="n">
+      <c r="G132" t="n">
+        <v>0.003846154038018522</v>
+      </c>
+      <c r="H132" t="n">
         <v>0.1119654605316557</v>
       </c>
-      <c r="F132" t="n">
+      <c r="I132" t="n">
         <v>0.5003799282718968</v>
       </c>
-      <c r="G132" t="n">
+      <c r="J132" t="n">
         <v>0.557249464368394</v>
       </c>
     </row>
@@ -3742,21 +4936,30 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.167367744990359</v>
+        <v>0.006388383263132669</v>
       </c>
       <c r="C133" t="n">
+        <v>0.004146913838165765</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0.003366134586809148</v>
+      </c>
+      <c r="E133" t="n">
         <v>0.2409045812685175</v>
       </c>
-      <c r="D133" t="n">
+      <c r="F133" t="n">
         <v>0.01106440680406851</v>
       </c>
-      <c r="E133" t="n">
+      <c r="G133" t="n">
+        <v>0.003693621613677398</v>
+      </c>
+      <c r="H133" t="n">
         <v>0.1177586007921525</v>
       </c>
-      <c r="F133" t="n">
+      <c r="I133" t="n">
         <v>0.4238430948367942</v>
       </c>
-      <c r="G133" t="n">
+      <c r="J133" t="n">
         <v>0.4629141371344831</v>
       </c>
     </row>
@@ -3767,21 +4970,30 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.1998892880149342</v>
+        <v>0.007674563006729127</v>
       </c>
       <c r="C134" t="n">
+        <v>0.005478314005643843</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0.004871796609855497</v>
+      </c>
+      <c r="E134" t="n">
         <v>0.2878850124589076</v>
       </c>
-      <c r="D134" t="n">
+      <c r="F134" t="n">
         <v>0.01373491603961786</v>
       </c>
-      <c r="E134" t="n">
+      <c r="G134" t="n">
+        <v>0.004106299196954367</v>
+      </c>
+      <c r="H134" t="n">
         <v>0.119569703291524</v>
       </c>
-      <c r="F134" t="n">
+      <c r="I134" t="n">
         <v>0.5083846102510234</v>
       </c>
-      <c r="G134" t="n">
+      <c r="J134" t="n">
         <v>0.5719472399957201</v>
       </c>
     </row>
@@ -3792,21 +5004,30 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.1758044557660635</v>
+        <v>0.006620248232879399</v>
       </c>
       <c r="C135" t="n">
+        <v>0.004417512946055547</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0.003703289200254588</v>
+      </c>
+      <c r="E135" t="n">
         <v>0.2531609563444053</v>
       </c>
-      <c r="D135" t="n">
+      <c r="F135" t="n">
         <v>0.01197811034630353</v>
       </c>
-      <c r="E135" t="n">
+      <c r="G135" t="n">
+        <v>0.004823100579913155</v>
+      </c>
+      <c r="H135" t="n">
         <v>0.1204340812508732</v>
       </c>
-      <c r="F135" t="n">
+      <c r="I135" t="n">
         <v>0.4472771068549365</v>
       </c>
-      <c r="G135" t="n">
+      <c r="J135" t="n">
         <v>0.4873732384796652</v>
       </c>
     </row>
@@ -3817,21 +5038,30 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.1897590654555214</v>
+        <v>0.007407981952371976</v>
       </c>
       <c r="C136" t="n">
+        <v>0.005121323730962459</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0.004376367735074931</v>
+      </c>
+      <c r="E136" t="n">
         <v>0.2734055741821582</v>
       </c>
-      <c r="D136" t="n">
+      <c r="F136" t="n">
         <v>0.01452972694938785</v>
       </c>
-      <c r="E136" t="n">
+      <c r="G136" t="n">
+        <v>0.003179931860605986</v>
+      </c>
+      <c r="H136" t="n">
         <v>0.1393548514637678</v>
       </c>
-      <c r="F136" t="n">
+      <c r="I136" t="n">
         <v>0.4607714303321129</v>
       </c>
-      <c r="G136" t="n">
+      <c r="J136" t="n">
         <v>0.5390081158294295</v>
       </c>
     </row>
@@ -3842,21 +5072,30 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.1600241842547316</v>
+        <v>0.006344872231364166</v>
       </c>
       <c r="C137" t="n">
+        <v>0.004030268901750724</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.003219609379090081</v>
+      </c>
+      <c r="E137" t="n">
         <v>0.2304446391300324</v>
       </c>
-      <c r="D137" t="n">
+      <c r="F137" t="n">
         <v>0.0113448903733558</v>
       </c>
-      <c r="E137" t="n">
+      <c r="G137" t="n">
+        <v>0.003455231355003297</v>
+      </c>
+      <c r="H137" t="n">
         <v>0.1310879425532902</v>
       </c>
-      <c r="F137" t="n">
+      <c r="I137" t="n">
         <v>0.3893955784170664</v>
       </c>
-      <c r="G137" t="n">
+      <c r="J137" t="n">
         <v>0.4398600836086127</v>
       </c>
     </row>

</xml_diff>